<commit_message>
XLS: sync W1-W3 Status sheet from DELIVERY-PLAN-STATUS.md (2026-07-24)
Bumps the stale 2026-07-21 completion %s to current: Movers/Heatmap/Dashboard/
Macro&VIX/IPOs/Commentary/Sector-Themes/Portfolio/Watchlist/Empty-states/Stock-
Detail/Fear&Greed all → 100%. 10-quarter EPS recapped 100%→90% (actuals complete;
estimate overlay needs Polygon's Benzinga add-on). Rollup: 17 of 18 at 100%,
avg ~99%. Refreshed the title date + summary.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Doc/MarketCatalyst.ai_weekly_deliverables_Plan.xlsx
+++ b/Doc/MarketCatalyst.ai_weekly_deliverables_Plan.xlsx
@@ -691,14 +691,14 @@
     <row r="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>MarketCatalyst — W1–W3 + Milestone 1/2 Status (refreshed 2026-07-21)</t>
+          <t>MarketCatalyst — W1–W3 + Milestone 1/2 Status (refreshed 2026-07-24)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" s="27">
       <c r="A2" s="37" t="inlineStr">
         <is>
-          <t>ALL DEPLOYED to production (single project market-catalyst-502415). Overall avg completion 93% across 18 deliverables; 5 at 100%. Remaining gaps: deferred AI (your choice), vendor-blocked features, and heavier data backfills.</t>
+          <t>ALL DEPLOYED to production (single project market-catalyst-502415). Refreshed 2026-07-24 from DELIVERY-PLAN-STATUS.md: avg ~99% across 18 W1–W3 deliverables; 17 at 100%. The ONLY sub-100% item is 10-quarter EPS history (90%) — its actuals are complete, but the estimate overlay needs Polygon's Benzinga add-on. Remaining plan-wide gaps: deferred AI (Anthropic/OpenRouter key), and vendor-blocked depth (options greeks, per-firm analyst events).</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="D9" s="34" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E9" s="33" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="F9" s="33" t="inlineStr">
         <is>
-          <t>Catalyst column is a news-presence heuristic, not true event attribution. MA-posture / week% / tech-context are real &amp; live.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="33" t="inlineStr">
         <is>
-          <t>Correlate each mover with same-day news/earnings/analyst events for a true catalyst; else the honest heuristic stands.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -942,7 +942,7 @@
       </c>
       <c r="D10" s="35" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E10" s="33" t="inlineStr">
@@ -952,12 +952,12 @@
       </c>
       <c r="F10" s="33" t="inlineStr">
         <is>
-          <t>No S&amp;P 500 constituent list, so the dead 'S&amp;P 500' tab was repurposed to a real Day%/Week% heat toggle. Tooltip reads live companies.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="33" t="inlineStr">
         <is>
-          <t>Source an S&amp;P 500 membership list from a vendor to add a genuine index filter as a third view.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
       </c>
       <c r="D11" s="34" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E11" s="33" t="inlineStr">
@@ -989,12 +989,12 @@
       </c>
       <c r="F11" s="33" t="inlineStr">
         <is>
-          <t>Recaps card still a .txt stub (needs R28 recap job). 'What Matters Now' AI card is a labeled placeholder (AI deferred by your decision). Internals + F&amp;G history now live.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G11" s="33" t="inlineStr">
         <is>
-          <t>Build the R28 Recaps EOD job; wire Anthropic (R34) for the AI card when AI is enabled.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="D12" s="35" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E12" s="33" t="inlineStr">
@@ -1026,12 +1026,12 @@
       </c>
       <c r="F12" s="33" t="inlineStr">
         <is>
-          <t>VIX shown via VIXY ETN proxy (plan has no spot-VIX) — labeled. Econ-calendar fallback now carries a Sample badge.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="33" t="inlineStr">
         <is>
-          <t>Upgrade the data plan for spot VIX if exact levels matter; otherwise the labeled proxy is fine.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="D13" s="35" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E13" s="33" t="inlineStr">
@@ -1063,12 +1063,12 @@
       </c>
       <c r="F13" s="33" t="inlineStr">
         <is>
-          <t>Aftermarket returns now REAL for IPOs listed within the 45-day sync window (current price, day-1 close, return-since-offer via Polygon aggs). Marquee historical names still use the sample showcase.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G13" s="33" t="inlineStr">
         <is>
-          <t>Add a one-time backfill of notable recent IPOs (fetch aggs once) to replace the sample showcase table.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D14" s="34" t="inlineStr">
         <is>
-          <t>82%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E14" s="33" t="inlineStr">
@@ -1100,12 +1100,12 @@
       </c>
       <c r="F14" s="33" t="inlineStr">
         <is>
-          <t>Main feed is live; Premarket/After-hours/General cards are static copy — now carry a Sample badge, but not yet live-driven.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="33" t="inlineStr">
         <is>
-          <t>Derive premarket/after-hours items from news publishedAt timestamps to make them live.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="D15" s="34" t="inlineStr">
         <is>
-          <t>82%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E15" s="33" t="inlineStr">
@@ -1137,12 +1137,12 @@
       </c>
       <c r="F15" s="33" t="inlineStr">
         <is>
-          <t>Live prices overlay per ticker; unmatched tickers show frozen sample prices — now flagged with a Sample badge.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G15" s="33" t="inlineStr">
         <is>
-          <t>Expand universe coverage for theme constituents so fewer rows fall back to frozen prices.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="D17" s="34" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E17" s="33" t="inlineStr">
@@ -1211,12 +1211,12 @@
       </c>
       <c r="F17" s="33" t="inlineStr">
         <is>
-          <t>Real holdings + live prices + P&amp;L work; dashboard fake $128,430 fallback removed. Pre-signin Portfolio screen still shows demo data.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="33" t="inlineStr">
         <is>
-          <t>Label the pre-signin demo portfolio, or gate behind an 'add your first holding' empty state.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D18" s="34" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E18" s="33" t="inlineStr">
@@ -1248,12 +1248,12 @@
       </c>
       <c r="F18" s="33" t="inlineStr">
         <is>
-          <t>Persistence + live prices complete. 'AI summary' is a template (AI deferred by your decision).</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G18" s="33" t="inlineStr">
         <is>
-          <t>Wire Anthropic (R34) for a real summary when AI is enabled; until then it's a heuristic summary.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="D19" s="34" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E19" s="33" t="inlineStr">
@@ -1285,12 +1285,12 @@
       </c>
       <c r="F19" s="33" t="inlineStr">
         <is>
-          <t>SampleBadge applied to the main silent-fallback surfaces (Recap, Themes, Macro, Commentary, Analyst, Insider). A few minor sub-cards remain unlabeled.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G19" s="33" t="inlineStr">
         <is>
-          <t>Apply &lt;SampleBadge&gt; to the last remaining fallbacks (a few dashboard sub-cards) for full coverage.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="D21" s="34" t="inlineStr">
         <is>
-          <t>80%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E21" s="33" t="inlineStr">
@@ -1329,12 +1329,12 @@
       </c>
       <c r="F21" s="33" t="inlineStr">
         <is>
-          <t>Financials, 10-quarter EPS, pivots, SMA rows all REAL. Remaining gap is data not fabrication: 1D/1W need intraday bars (not synced); 5Y needs 5yr history (only ~300d).</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G21" s="33" t="inlineStr">
         <is>
-          <t>Add an intraday-bars sync for 1D/1W; extend the ohlcv_bars backfill to 5 years for the 5Y chart.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="D22" s="35" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E22" s="33" t="inlineStr">
@@ -1366,12 +1366,12 @@
       </c>
       <c r="F22" s="33" t="inlineStr">
         <is>
-          <t>Gauge value uses the full 4-component composite; the HISTORY sparkline is a breadth-derived proxy (no long history for SPY/TLT/VIXY).</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G22" s="33" t="inlineStr">
         <is>
-          <t>Backfill SPY/TLT/VIXY price history so F&amp;G history uses the full composite instead of breadth alone.</t>
+          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="D23" s="35" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="E23" s="33" t="inlineStr">
@@ -1403,16 +1403,15 @@
       </c>
       <c r="F23" s="33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Estimate overlay (actual-vs-estimate beat/miss) has no redistributable source on Polygon Stocks Starter. The 10 quarters of EPS ACTUALS are 100% and now also drive Quarterly/Yearly EPS &amp; Sales + Income-statement tabs (8 annual years added 2026-07-24).</t>
         </is>
       </c>
       <c r="G23" s="33" t="inlineStr">
         <is>
-          <t>Complete — 10 real actual quarters (Polygon /vX) + estimate line now filled from Finnhub /calendar/earnings on top of FMP.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24"/>
+          <t>Purchase Polygon's Benzinga Earnings &amp; Estimates add-on to ship forward EPS + %-surprise. Cannot reach 100% on current data.</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
       <c r="A25" s="39" t="inlineStr">
         <is>
@@ -1421,7 +1420,7 @@
       </c>
       <c r="C25" s="40" t="inlineStr">
         <is>
-          <t>18 deliverables · avg 93% · 6 at 100%</t>
+          <t>18 deliverables · avg ~99% · 17 at 100% · 1 at 90% (10-qtr EPS — estimate overlay needs Benzinga)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: add Screen·Feature column to delivery status; mirror full table into xlsx sheet 1
Adds a 'Screen · Feature' column mapping each requirement to the app screen it
powers, and copies the full row-by-row table (10 columns × 36 rows) into the
Excel workbook's first sheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Doc/MarketCatalyst.ai_weekly_deliverables_Plan.xlsx
+++ b/Doc/MarketCatalyst.ai_weekly_deliverables_Plan.xlsx
@@ -6,7 +6,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="60" yWindow="660" windowWidth="30240" windowHeight="17740" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W1-W3 Status (updated)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Row-by-Row Status" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Plan (W1-W10)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -108,8 +108,30 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -181,8 +203,18 @@
         <fgColor rgb="00EAF0F7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -219,11 +251,25 @@
         <color rgb="00D0D0D0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -311,6 +357,27 @@
     <xf numFmtId="0" fontId="14" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -676,759 +743,1963 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="27" min="1" max="1"/>
-    <col width="9" customWidth="1" style="27" min="2" max="2"/>
-    <col width="34" customWidth="1" style="27" min="3" max="3"/>
-    <col width="12" customWidth="1" style="27" min="4" max="4"/>
-    <col width="34" customWidth="1" style="27" min="5" max="5"/>
-    <col width="48" customWidth="1" style="27" min="6" max="6"/>
-    <col width="48" customWidth="1" style="27" min="7" max="7"/>
+    <col width="6" customWidth="1" style="27" min="1" max="1"/>
+    <col width="6" customWidth="1" style="27" min="2" max="2"/>
+    <col width="6" customWidth="1" style="27" min="3" max="3"/>
+    <col width="30" customWidth="1" style="27" min="4" max="4"/>
+    <col width="18" customWidth="1" style="27" min="5" max="5"/>
+    <col width="34" customWidth="1" style="27" min="6" max="6"/>
+    <col width="28" customWidth="1" style="27" min="7" max="7"/>
+    <col width="9" customWidth="1" style="27" min="8" max="8"/>
+    <col width="30" customWidth="1" style="27" min="9" max="9"/>
+    <col width="70" customWidth="1" style="27" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="30" t="inlineStr">
-        <is>
-          <t>MarketCatalyst — W1–W3 + Milestone 1/2 Status (refreshed 2026-07-24)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="44" customHeight="1" s="27">
-      <c r="A2" s="37" t="inlineStr">
-        <is>
-          <t>ALL DEPLOYED to production (single project market-catalyst-502415). Refreshed 2026-07-24 from DELIVERY-PLAN-STATUS.md: avg ~99% across 18 W1–W3 deliverables; 17 at 100%. The ONLY sub-100% item is 10-quarter EPS history (90%) — its actuals are complete, but the estimate overlay needs Polygon's Benzinga add-on. Remaining plan-wide gaps: deferred AI (Anthropic/OpenRouter key), and vendor-blocked depth (options greeks, per-firm analyst events).</t>
+    <row r="1" ht="22" customHeight="1" s="27">
+      <c r="A1" s="41" t="inlineStr">
+        <is>
+          <t>MarketCatalyst — Delivery Status (row-by-row) · exact copy of DELIVERY-PLAN-STATUS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1" s="27">
+      <c r="A2" s="42" t="inlineStr">
+        <is>
+          <t>State sync 2026-07-24 · all 36 rows · Polygon/Massive is the only vendor served to users. 'Screen · Feature' = the app screen this row powers (— for infra/enabler/AI-unwired rows).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1" s="27">
+      <c r="A3" s="43" t="inlineStr">
+        <is>
+          <t>Row</t>
+        </is>
+      </c>
+      <c r="B3" s="43" t="inlineStr">
+        <is>
+          <t>Wk</t>
+        </is>
+      </c>
+      <c r="C3" s="43" t="inlineStr">
+        <is>
+          <t>Due</t>
+        </is>
+      </c>
+      <c r="D3" s="43" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="E3" s="43" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="F3" s="43" t="inlineStr">
+        <is>
+          <t>API URL</t>
+        </is>
+      </c>
+      <c r="G3" s="43" t="inlineStr">
+        <is>
+          <t>Screen · Feature</t>
+        </is>
+      </c>
+      <c r="H3" s="43" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I3" s="43" t="inlineStr">
+        <is>
+          <t>What's NOT done</t>
+        </is>
+      </c>
+      <c r="J3" s="43" t="inlineStr">
+        <is>
+          <t>Reason</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="32" t="inlineStr">
-        <is>
-          <t>Rel / Week</t>
-        </is>
-      </c>
-      <c r="B4" s="32" t="inlineStr">
-        <is>
-          <t>Dates</t>
-        </is>
-      </c>
-      <c r="C4" s="32" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
-        </is>
-      </c>
-      <c r="D4" s="32" t="inlineStr">
-        <is>
-          <t>Completion %</t>
-        </is>
-      </c>
-      <c r="E4" s="32" t="inlineStr">
-        <is>
-          <t>Pushed to Production?</t>
-        </is>
-      </c>
-      <c r="F4" s="32" t="inlineStr">
-        <is>
-          <t>Reason (if not 100%)</t>
-        </is>
-      </c>
-      <c r="G4" s="32" t="inlineStr">
-        <is>
-          <t>Suggestion to reach 100%</t>
+      <c r="A4" s="44" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B4" s="44" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="C4" s="44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D4" s="45" t="inlineStr">
+        <is>
+          <t>FOUNDATION: deploy FE+BE 24/7, Blaze, service-account, indexes+TTL</t>
+        </is>
+      </c>
+      <c r="E4" s="45" t="inlineStr">
+        <is>
+          <t>Firebase / Cloud Run</t>
+        </is>
+      </c>
+      <c r="F4" s="45" t="inlineStr">
+        <is>
+          <t>— (infra: Hosting + Cloud Run + Firestore)</t>
+        </is>
+      </c>
+      <c r="G4" s="45" t="inlineStr">
+        <is>
+          <t>— *(infra)*</t>
+        </is>
+      </c>
+      <c r="H4" s="44" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I4" s="45" t="inlineStr">
+        <is>
+          <t>— (R5 scope fully delivered; the Polygon key rotation + rules-drift items are R49's scope, separately tracked — not a dependency of this row)</t>
+        </is>
+      </c>
+      <c r="J4" s="45" t="inlineStr">
+        <is>
+          <t>✅ Complete 2026-07-23. Every element of R5's stated scope is delivered and verified: deploy FE+BE (FE marketcatalyst.web.app; worker rev 00035-d74 + public market-catalyst-live), 24/7 (21 Cloud Scheduler jobs ENABLED and firing on schedule — sync-companies 2026-07-23 06:00 UTC, sync-news 20:30 UTC, sync-market-movers 22:00 UTC — all matching their crons; scheduler-invoker SA present), Blaze (Cloud Run + Scheduler operating), service-account (runtime SA least-privilege: datastore.user+secretAccessor), indexes (deployed), TTL (not possible on ISO-string dates → substituted with the in-code retention module, weekly prune, RETENTION_DRY_RUN=false). Backend is browser-reachable and CORS-verified. Security follow-ups live in R49, not here.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="33" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B5" s="46" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="B5" s="33" t="inlineStr">
-        <is>
-          <t>06 Jul</t>
-        </is>
-      </c>
-      <c r="C5" s="33" t="inlineStr">
-        <is>
-          <t>FOUNDATION: deploy FE+BE 24/7, Blaze, service-account, indexes+TTL</t>
-        </is>
-      </c>
-      <c r="D5" s="35" t="inlineStr">
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D5" s="47" t="inlineStr">
+        <is>
+          <t>Feature-flag system (feature_flags doc, per-release FF_* toggles)</t>
+        </is>
+      </c>
+      <c r="E5" s="47" t="inlineStr">
+        <is>
+          <t>— (internal)</t>
+        </is>
+      </c>
+      <c r="F5" s="47" t="inlineStr">
+        <is>
+          <t>— (Firestore feature_flags)</t>
+        </is>
+      </c>
+      <c r="G5" s="47" t="inlineStr">
+        <is>
+          <t>— *(internal)*</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="E5" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F5" s="33" t="inlineStr">
+      <c r="I5" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G5" s="33" t="inlineStr">
-        <is>
-          <t>Complete — retention activated (RETENTION_DRY_RUN=false, 0 eligible verified). Native TTL impossible (ISO-string dates); in-code retention enforces it. Runtime SA least-privilege.</t>
+      <c r="J5" s="47" t="inlineStr">
+        <is>
+          <t>Built 2026-07-21: registry + service + API + UI provider/Gate + nav &amp; screen gating. Deployed rev 00017; feature_flags/default auto-seeded 25 flags in prod; resolver verified (default→env→Firestore, fail-open). Extended 2026-07-22 with a SECOND, independent gating layer — per-plan entitlements (src/plans/plans.registry.ts, 16 keys × 3 plans) plus an admin UI to edit them per plan (public/admin/console.html feature editor, writing plans/{id}.featureFlags under a rules constraint that permits only featureFlags+updatedAt). The two layers are deliberately NOT merged: FF_* answers *"is it built and shipped?"* → "coming soon"; entitlements answer *"may this tier use it?"* → "upgrade to unlock". Merging them would make an unbuilt feature masquerade as a paywall. Scope exceeded, not just met</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="44" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="B6" s="44" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="B6" s="33" t="inlineStr">
-        <is>
-          <t>06 Jul</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>Feature-flag system (feature_flags doc, per-release FF_* toggles)</t>
-        </is>
-      </c>
-      <c r="D6" s="35" t="inlineStr">
+      <c r="C6" s="44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D6" s="45" t="inlineStr">
+        <is>
+          <t>Project setup: Firebase, Polygon sub + keys, data-source verification</t>
+        </is>
+      </c>
+      <c r="E6" s="45" t="inlineStr">
+        <is>
+          <t>Polygon (Massive)</t>
+        </is>
+      </c>
+      <c r="F6" s="45" t="inlineStr">
+        <is>
+          <t>— (key/entitlement verification)</t>
+        </is>
+      </c>
+      <c r="G6" s="45" t="inlineStr">
+        <is>
+          <t>— *(setup)*</t>
+        </is>
+      </c>
+      <c r="H6" s="44" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="E6" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F6" s="33" t="inlineStr">
+      <c r="I6" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G6" s="33" t="inlineStr">
-        <is>
-          <t>Complete — resolver + API + UI gating live; doc auto-seeded 25 flags; read rule deployed.</t>
+      <c r="J6" s="45" t="inlineStr">
+        <is>
+          <t>Complete — all keys present and verified</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="33" t="inlineStr">
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t>R8</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="B7" s="33" t="inlineStr">
-        <is>
-          <t>06 Jul</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="inlineStr">
-        <is>
-          <t>Project setup: Firebase, Polygon subscription + API keys, verification</t>
-        </is>
-      </c>
-      <c r="D7" s="35" t="inlineStr">
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D7" s="47" t="inlineStr">
+        <is>
+          <t>Run all sync jobs once; verify sync_meta + ops dashboard</t>
+        </is>
+      </c>
+      <c r="E7" s="47" t="inlineStr">
+        <is>
+          <t>multiple (all sync jobs)</t>
+        </is>
+      </c>
+      <c r="F7" s="47" t="inlineStr">
+        <is>
+          <t>— (21 jobs; see per-row endpoints)</t>
+        </is>
+      </c>
+      <c r="G7" s="47" t="inlineStr">
+        <is>
+          <t>— *(all sync jobs)*</t>
+        </is>
+      </c>
+      <c r="H7" s="46" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="E7" s="33" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="F7" s="33" t="inlineStr">
+      <c r="I7" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G7" s="33" t="inlineStr">
-        <is>
-          <t>Complete.</t>
+      <c r="J7" s="47" t="inlineStr">
+        <is>
+          <t>21/21 jobs run, sync_meta populated, monitor UI live</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="inlineStr">
+      <c r="A8" s="44" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="B8" s="33" t="inlineStr">
-        <is>
-          <t>06 Jul</t>
-        </is>
-      </c>
-      <c r="C8" s="33" t="inlineStr">
-        <is>
-          <t>Run all sync jobs once; verify sync_meta + ops dashboard</t>
-        </is>
-      </c>
-      <c r="D8" s="35" t="inlineStr">
+      <c r="C8" s="44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D8" s="45" t="inlineStr">
+        <is>
+          <t>Market Movers live (gainers/losers/unusual-vol/RVol/filter)</t>
+        </is>
+      </c>
+      <c r="E8" s="45" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F8" s="45" t="inlineStr">
+        <is>
+          <t>/v2/snapshot/…/{gainers,losers} + /v2/aggs/grouped/locale/us/market/stocks/{date}</t>
+        </is>
+      </c>
+      <c r="G8" s="45" t="inlineStr">
+        <is>
+          <t>Movers · gainers / losers / unusual-vol table</t>
+        </is>
+      </c>
+      <c r="H8" s="44" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I8" s="45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J8" s="45" t="inlineStr">
+        <is>
+          <t>✅ 2026-07-21: MA-posture (real SMA50/200), week% (real 5-session change), tech-context (RSI/MACD/RS/RVOL) now live — added SMA/week fields to technical-indicators.job (rev 00019, ran for 238 tickers); catalyst now flags tickers with recent synced news ⬆ 100% on 2026-07-23: the catalyst field is now strictly honest — 'Recent news' (a real recent Polygon article exists for the ticker, via companies.newsCount) or 'No known catalyst'. The fabricated fallback to the hardcoded mock label ('Earnings beat', 'Guidance raise') was removed from the Movers screen, the Dashboard movers widget and the mover drawer — no row asserts an invented catalyst. Everything on this row is now Polygon-sourced with zero fabrication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="46" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D9" s="47" t="inlineStr">
+        <is>
+          <t>Market Heatmap live (sector %, tiles, summary)</t>
+        </is>
+      </c>
+      <c r="E9" s="47" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F9" s="47" t="inlineStr">
+        <is>
+          <t>/v2/aggs/grouped/locale/us/market/stocks/{date} (11 SPDR sector-ETF proxies)</t>
+        </is>
+      </c>
+      <c r="G9" s="47" t="inlineStr">
+        <is>
+          <t>Heatmap · sector treemap + tiles</t>
+        </is>
+      </c>
+      <c r="H9" s="46" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I9" s="47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J9" s="47" t="inlineStr">
+        <is>
+          <t>✅ 2026-07-21: hover tooltip now reads live companies (price/RVOL/RS/MA-status); dead Stocks/S&amp;P-500 tab repurposed to a real Day%/Week% heat toggle (5-session change from technical-indicators.job, cap-weighted sector avg). S&amp;P-500 filter dropped — no constituent list available ⬆ 100% 2026-07-23: heatmap tiles now sample-labeled when no live sector data has synced; the dropped S&amp;P-500 filter was an out-of-scope extra (no constituent list on Starter), so the stated deliverable (sector %/tiles/summary) is fully met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="44" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="B10" s="44" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="C10" s="44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D10" s="45" t="inlineStr">
+        <is>
+          <t>Dashboard core widgets live (AI card → R19)</t>
+        </is>
+      </c>
+      <c r="E10" s="45" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F10" s="45" t="inlineStr">
+        <is>
+          <t>/v2/aggs/grouped/locale/us/market/stocks/{date} (market-breadth)</t>
+        </is>
+      </c>
+      <c r="G10" s="45" t="inlineStr">
+        <is>
+          <t>Dashboard · core widgets (Market Pulse, internals, VIX)</t>
+        </is>
+      </c>
+      <c r="H10" s="44" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I10" s="45" t="inlineStr">
+        <is>
+          <t>AI card → R35 (Anthropic); Recaps → R28 — both separately tracked, not this row</t>
+        </is>
+      </c>
+      <c r="J10" s="45" t="inlineStr">
+        <is>
+          <t>✅ 2026-07-21: Market Internals + F&amp;G history now live from new market-breadth.job (176 days backfilled); VIX/Portfolio fake fallbacks removed (show — when absent) ⬆ 100% of the core-widget scope 2026-07-23. All dashboard widgets are live from Polygon; the 'What Matters Now' AI card is tracked in R35 (Anthropic — your planned purchase) and the Recaps card in R28, neither part of this row's widget deliverable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="B11" s="46" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="C11" s="46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D11" s="47" t="inlineStr">
+        <is>
+          <t>Macro &amp; VIX live (econ calendar + dividends + VIX/yields)</t>
+        </is>
+      </c>
+      <c r="E11" s="47" t="inlineStr">
+        <is>
+          <t>Polygon + FRED (US-gov)</t>
+        </is>
+      </c>
+      <c r="F11" s="47" t="inlineStr">
+        <is>
+          <t>Polygon /fed/v1/treasury-yields + VIXY via /v2/aggs; FRED macro series (FredService). Not Finnhub.</t>
+        </is>
+      </c>
+      <c r="G11" s="47" t="inlineStr">
+        <is>
+          <t>Macro · VIX card, 10-yr yield, dividends</t>
+        </is>
+      </c>
+      <c r="H11" s="46" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I11" s="47" t="inlineStr">
+        <is>
+          <t>True spot VIX needs the Polygon Indices add-on (a purchase); VIXY proxy is the delivered, labeled solution</t>
+        </is>
+      </c>
+      <c r="J11" s="47" t="inlineStr">
+        <is>
+          <t>✅ 2026-07-21: Macro VIX card live via market_indices VIXY; dividend Month tab from live dividends. ⚠️ Correctness fix 2026-07-22 — the 10-year yield was previously WRONG, not merely proxied. market-indices.job.ts was publishing the TLT ETF price under the label "US10Y". TLT moves *inversely* to the yield it was labelled as, so the card showed the yield falling when it was rising. Now sourced from Polygon /fed/v1/treasury-yields — the real Treasury yield, isProxy:false, unit:"percent". Also new: dividend_history/{ticker} (241 docs) carrying full payment history, annual totals, TTM, derived yield, 5y CAGR and increase streak; and splits/{ticker} (241 docs) ⬆ 100% 2026-07-23: VIXY is the delivered, honestly-labeled (isProxy:true) proxy — consistent with the ETF proxies used for every index tile in this app. Spot VIX (I:VIX → 403) would need the Polygon Indices add-on, a future purchase like AI, not a gap in the delivered solution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="44" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="C12" s="44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D12" s="45" t="inlineStr">
+        <is>
+          <t>IPOs live (calendar + offer price)</t>
+        </is>
+      </c>
+      <c r="E12" s="45" t="inlineStr">
+        <is>
+          <t>Polygon (only)</t>
+        </is>
+      </c>
+      <c r="F12" s="45" t="inlineStr">
+        <is>
+          <t>/vX/reference/ipos. Finnhub fallback removed — not redistribution-licensed; prod already ran fallback=none.</t>
+        </is>
+      </c>
+      <c r="G12" s="45" t="inlineStr">
+        <is>
+          <t>IPOs · IPO calendar + aftermarket perf</t>
+        </is>
+      </c>
+      <c r="H12" s="44" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I12" s="45" t="inlineStr">
+        <is>
+          <t>SPAC units / brand-new tickers with no Polygon bars show "—" (honest, not mock)</t>
+        </is>
+      </c>
+      <c r="J12" s="45" t="inlineStr">
+        <is>
+          <t>⬆ Corrected 2026-07-23 — the 'falls back to mock' note was stale. ipos.job.ts already derives day-1 and since-IPO returns from Polygon /v2/aggs (getAggsRange) — verified live: 40/52 IPO docs carry real aftermarket performance. The mock RECENT_IPOS renders only when the live collection is empty (it isn't). Polygon-only, no non-redistributable data. ⬆ 100% 2026-07-23.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="46" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="B13" s="46" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="C13" s="46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D13" s="47" t="inlineStr">
+        <is>
+          <t>Commentary/News live (aggregated feed + tags + drawer)</t>
+        </is>
+      </c>
+      <c r="E13" s="47" t="inlineStr">
+        <is>
+          <t>Polygon (only)</t>
+        </is>
+      </c>
+      <c r="F13" s="47" t="inlineStr">
+        <is>
+          <t>/v2/reference/news. Finnhub dropped from the news feed — not redistribution-licensed (was NEWS_SOURCE=aggregate).</t>
+        </is>
+      </c>
+      <c r="G13" s="47" t="inlineStr">
+        <is>
+          <t>Commentary · aggregated news feed</t>
+        </is>
+      </c>
+      <c r="H13" s="46" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I13" s="47" t="inlineStr">
+        <is>
+          <t>Narrative "before the bell / after the close" briefs are AI content → R35 (Anthropic), honestly SampleBadge-labeled</t>
+        </is>
+      </c>
+      <c r="J13" s="47" t="inlineStr">
+        <is>
+          <t>Those sub-feeds have no live source; main feed is live ⬆ 100% of the DATA scope 2026-07-23: the news feed (Polygon /v2/reference/news) and extended-hours moves (Polygon /v3/snapshot via useExtendedHours) are live; the two narrative brief cards are AI-generated content, labeled and tracked under R35 (Anthropic). No non-AI gap remains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="44" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="C14" s="44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D14" s="45" t="inlineStr">
+        <is>
+          <t>Sector Themes live (per-stock prices + theme perf)</t>
+        </is>
+      </c>
+      <c r="E14" s="45" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F14" s="45" t="inlineStr">
+        <is>
+          <t>/v3/reference/tickers (companies prices)</t>
+        </is>
+      </c>
+      <c r="G14" s="45" t="inlineStr">
+        <is>
+          <t>Themes · sector-theme baskets</t>
+        </is>
+      </c>
+      <c r="H14" s="44" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I14" s="45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J14" s="45" t="inlineStr">
+        <is>
+          <t>Theme baskets are static config (fine); prices live when matched ⬆ 100% 2026-07-23: matched tickers show live Polygon prices; unmatched (outside the synced universe) are SampleBadge-labeled with a live/total count. Theme baskets are static config by design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="46" t="inlineStr">
+        <is>
+          <t>R17</t>
+        </is>
+      </c>
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="C15" s="46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D15" s="47" t="inlineStr">
+        <is>
+          <t>Company-name search (nameLower/tokens)</t>
+        </is>
+      </c>
+      <c r="E15" s="47" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F15" s="47" t="inlineStr">
+        <is>
+          <t>/v3/reference/tickers</t>
+        </is>
+      </c>
+      <c r="G15" s="47" t="inlineStr">
+        <is>
+          <t>Search (⌘K / shell) · company-name search</t>
+        </is>
+      </c>
+      <c r="H15" s="46" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I15" s="47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J15" s="47" t="inlineStr">
+        <is>
+          <t>ticker-universe writes nameLower/searchTokens; ⌘K search live ⬆ 100% 2026-07-23: company-name search is live over the full ticker universe (nameLower/searchTokens). ⬆ 2026-07-23: ⌘K search results now overlay live delayed prices (Polygon /live/snapshot via useSnapshotQuotes, polled only while the palette is open) on top of the EOD companies price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="44" t="inlineStr">
+        <is>
+          <t>R19</t>
+        </is>
+      </c>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="C16" s="44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D16" s="45" t="inlineStr">
+        <is>
+          <t>Portfolio Pulse live (holdings + prices + P&amp;L + totals)</t>
+        </is>
+      </c>
+      <c r="E16" s="45" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F16" s="45" t="inlineStr">
+        <is>
+          <t>/v3/snapshot · /v2/snapshot (holding prices)</t>
+        </is>
+      </c>
+      <c r="G16" s="45" t="inlineStr">
+        <is>
+          <t>Portfolio · holdings + prices + P&amp;L</t>
+        </is>
+      </c>
+      <c r="H16" s="44" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I16" s="45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J16" s="45" t="inlineStr">
+        <is>
+          <t>Real holdings + live prices + P&amp;L all work; fallback is cosmetic ⬆ 100% 2026-07-23: the Portfolio Pulse SCREEN uses real holdings + live Polygon prices + P&amp;L, sample-labeled when a holding is outside the synced universe. The $128,430 figure is on the pre-login MARKETING landing (page.tsx), a showcase — not the app. ⬆ 2026-07-23 — two upgrades. (1) Holding prices and the portfolio total (Σ shares×price) + day P&amp;L now track live delayed prices (Polygon /live/snapshot), not the once-a-day EOD write. (2) CRUD gap fixed: share quantity was hardcoded to 10 with no editor — added a Shares input to the add form and an editable position strip for the selected holding, both persisted to Firestore, so the total reflects real share counts. The $128,430 figure remains only on the marketing landing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="46" t="inlineStr">
+        <is>
+          <t>R20</t>
+        </is>
+      </c>
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="C17" s="46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D17" s="47" t="inlineStr">
+        <is>
+          <t>Watchlist live (persistence + prices + AI summary)</t>
+        </is>
+      </c>
+      <c r="E17" s="47" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F17" s="47" t="inlineStr">
+        <is>
+          <t>/v3/snapshot (watchlist prices)</t>
+        </is>
+      </c>
+      <c r="G17" s="47" t="inlineStr">
+        <is>
+          <t>Watchlist · prices + persistence</t>
+        </is>
+      </c>
+      <c r="H17" s="46" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I17" s="47" t="inlineStr">
+        <is>
+          <t>The "AI summary" is AI content → R39 (Anthropic); persistence + prices are done and labeled</t>
+        </is>
+      </c>
+      <c r="J17" s="47" t="inlineStr">
+        <is>
+          <t>AI intentionally deferred to R34/R39; persistence + prices done ⬆ 100% of the non-AI scope 2026-07-23: watchlist persistence + live Polygon prices are done and sample-labeled; the 'AI summary' is tracked under R39 (Anthropic — your planned purchase). ⬆ 2026-07-23: watchlist prices now overlay live delayed prices (Polygon /live/snapshot) on the EOD price. CRUD verified: add/remove persist via Firestore arrayUnion/arrayRemove on users/{uid}/watchlists/default. (AI summary still R39 — Anthropic.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="44" t="inlineStr">
+        <is>
+          <t>R21</t>
+        </is>
+      </c>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="C18" s="44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D18" s="45" t="inlineStr">
+        <is>
+          <t>Empty-states + graceful fallback polish (cross-screen)</t>
+        </is>
+      </c>
+      <c r="E18" s="45" t="inlineStr">
+        <is>
+          <t>— (cross-screen)</t>
+        </is>
+      </c>
+      <c r="F18" s="45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" s="45" t="inlineStr">
+        <is>
+          <t>— *(cross-screen empty states)*</t>
+        </is>
+      </c>
+      <c r="H18" s="44" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I18" s="45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J18" s="45" t="inlineStr">
+        <is>
+          <t>Only IPOs/Options/Insider label mock data; pattern not applied app-wide ⬆ 100% 2026-07-23: the sample-labeling pattern is now applied across every W1–W3 data screen — movers, screener, portfolio, watchlist and heatmap gained a &lt;SampleBadge&gt; (shown when data isn't fully live), joining the already-labeled commentary, earnings, insider, macro, recap, themes and ipos. No W1–W3 screen silently shows mock. (analyst/options/stock are labeled within their own rows R41/R32/R24.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="46" t="inlineStr">
+        <is>
+          <t>R23</t>
+        </is>
+      </c>
+      <c r="B19" s="46" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C19" s="46" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D19" s="47" t="inlineStr">
+        <is>
+          <t>ENABLER: backfill ohlcv_bars + compute jobs</t>
+        </is>
+      </c>
+      <c r="E19" s="47" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F19" s="47" t="inlineStr">
+        <is>
+          <t>/v2/aggs/ticker/{sym}/range/1/day/… + /range/{5,30}/minute/…</t>
+        </is>
+      </c>
+      <c r="G19" s="47" t="inlineStr">
+        <is>
+          <t>— *(enabler; feeds Stock-detail charts)*</t>
+        </is>
+      </c>
+      <c r="H19" s="46" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="E8" s="33" t="inlineStr">
-        <is>
-          <t>✅ Yes</t>
-        </is>
-      </c>
-      <c r="F8" s="33" t="inlineStr">
+      <c r="I19" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="33" t="inlineStr">
-        <is>
-          <t>Complete — now 24 jobs (added financials, market-breadth, retention).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="33" t="inlineStr">
-        <is>
-          <t>W1</t>
-        </is>
-      </c>
-      <c r="B9" s="33" t="inlineStr">
-        <is>
-          <t>06 Jul</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="inlineStr">
-        <is>
-          <t>Market Movers live (gainers/losers/unusual-vol/RVol/filter)</t>
-        </is>
-      </c>
-      <c r="D9" s="34" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E9" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F9" s="33" t="inlineStr">
+      <c r="J19" s="47" t="inlineStr">
+        <is>
+          <t>Ahead of schedule — all 5 compute jobs green. Deepened 2026-07-22: ohlcv_bars now holds ~299,552 documents spanning the full 5-year window (was ~300 days). Raising the backfill constant alone did nothing — lastSyncedThrough only ever advances — so stock-history.job.ts gained an earliestSyncedFrom watermark that fills history backwards as well as forwards, clamped to the plan's rolling 5-year edge. vwap now persisted per bar. Also new: intraday_bars (474 docs, 5-min + 30-min, one doc per ticker/resolution holding an array of bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="44" t="inlineStr">
+        <is>
+          <t>R24</t>
+        </is>
+      </c>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C20" s="44" t="inlineStr">
+        <is>
+          <t>🔵→</t>
+        </is>
+      </c>
+      <c r="D20" s="45" t="inlineStr">
+        <is>
+          <t>Stock Detail live (charts/RSI-MACD/fundamentals/52-wk/consensus/news/insider)</t>
+        </is>
+      </c>
+      <c r="E20" s="45" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F20" s="45" t="inlineStr">
+        <is>
+          <t>/v2/aggs/ticker/{sym}/range/…, /vX/reference/financials, /v1/related-companies/{sym}</t>
+        </is>
+      </c>
+      <c r="G20" s="45" t="inlineStr">
+        <is>
+          <t>Stock detail · chart / RSI-MACD / financials / 52-wk / peers</t>
+        </is>
+      </c>
+      <c r="H20" s="44" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I20" s="45" t="inlineStr">
+        <is>
+          <t>Analyst consensus uses FMP (required — Polygon has no analyst product on Starter); true per-firm analyst actions → R41 (Benzinga add-on). AI thesis/risk block → R38 (Anthropic). Both separately tracked</t>
+        </is>
+      </c>
+      <c r="J20" s="45" t="inlineStr">
+        <is>
+          <t>⬆ Raised from 80% on 2026-07-22 — the previous entry mis-diagnosed the gap. The old note said 1D/1W needed intraday bars and 5Y needed 5-year history, implying a data-plan block. That was wrong: both were authorized on the existing Polygon Stocks Starter plan all along (intraday aggregates ✅, 5-year rolling history ✅ — re-probed live). It was a sync gap, not a plan gap — we simply had not pulled them. Now synced: intraday-bars.job.ts (new) feeds 1D/1W, and the 5-year backfill (R23) feeds 5Y. All 7 chart timeframes now read real bars via useChartBars. Also real: full financial statements, 52-wk high/low + %-from, SMA/EMA ladders (10/20/30/50/100/200), 90-point rsi14Series, VWAP, peers (/v1/related-companies), dividend yield + DPS. No synthetic timeframes remain ⬆ 100% 2026-07-23 — all remaining fabrications on the screen removed. Revenue (TTM) now = last 4 real quarters (Polygon financials); the dead finRows panel and its fabricated FCF/debt are gone; the 'recent EPS' rows and the EPS-surprise pane now read real fin.epsHistory (beat/miss only where a real estimate exists, else 'no est.'); the technical ratings are computed from real indicators — Moving Averages from price vs each real SMA/EMA, Oscillators from real RSI(14)+MACD; and a header &lt;SampleBadge&gt; flags any ticker outside the synced universe (covering the RSI/SMA/vol/pivot/52wk fallbacks). The analyst consensus panel is FMP-backed — kept per decision; it is a consensus snapshot, and per-firm upgrades/downgrades remain R41 (Benzinga). The AI thesis is R38 (Anthropic). Charts, RSI/MACD, full financial statements, 52-week, news and insider (SEC) were already live. ⬆ 2026-07-24 deepened (still 100%): the header price + chart now use the shared live-price subscription (delayed snapshot) instead of the once-a-day close, and the fundamentals gained Quarterly / Yearly tabs (annual financials). The TradingView compare surface was removed from the shipped page — the stock chart is now our own Polygon-backed CandleChart, last bar tracking the live price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="46" t="inlineStr">
+        <is>
+          <t>R25</t>
+        </is>
+      </c>
+      <c r="B21" s="46" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C21" s="46" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D21" s="47" t="inlineStr">
+        <is>
+          <t>Screener live (filters + Tech Rating + RVOL + growth/margin)</t>
+        </is>
+      </c>
+      <c r="E21" s="47" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F21" s="47" t="inlineStr">
+        <is>
+          <t>/v3/reference/tickers + /vX/reference/financials</t>
+        </is>
+      </c>
+      <c r="G21" s="47" t="inlineStr">
+        <is>
+          <t>Screener · filters + Tech Rating + RVOL</t>
+        </is>
+      </c>
+      <c r="H21" s="46" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I21" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="33" t="inlineStr">
-        <is>
-          <t>W1</t>
-        </is>
-      </c>
-      <c r="B10" s="33" t="inlineStr">
-        <is>
-          <t>06 Jul</t>
-        </is>
-      </c>
-      <c r="C10" s="33" t="inlineStr">
-        <is>
-          <t>Market Heatmap live (sector %, tiles, summary)</t>
-        </is>
-      </c>
-      <c r="D10" s="35" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E10" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F10" s="33" t="inlineStr">
+      <c r="J21" s="47" t="inlineStr">
+        <is>
+          <t>Core overlay from companies live; a few filters never implemented ⬆ 100% 2026-07-23: the three dead no-op filter checkboxes — Above 50 &amp; 200-DMA, RSI 40–70, Price &gt; $5 — are now wired to real companies technicals (price/sma50/sma200/rsi14 from technical-indicators.job), with save/restore + reset. No no-op filter remains; every control filters on real Polygon-derived data. Verified against prod: of 241 priced companies, 114 pass the DMA filter, 211 RSI 40–70, 239 price&gt;$5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="44" t="inlineStr">
+        <is>
+          <t>R26</t>
+        </is>
+      </c>
+      <c r="B22" s="44" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C22" s="44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D22" s="45" t="inlineStr">
+        <is>
+          <t>Dashboard Fear &amp; Greed gauge live</t>
+        </is>
+      </c>
+      <c r="E22" s="45" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F22" s="45" t="inlineStr">
+        <is>
+          <t>/v2/aggs/range (SPY/TLT/VIXY) + /v2/aggs/grouped (breadth)</t>
+        </is>
+      </c>
+      <c r="G22" s="45" t="inlineStr">
+        <is>
+          <t>Dashboard · Fear &amp; Greed gauge</t>
+        </is>
+      </c>
+      <c r="H22" s="44" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I22" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G10" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="33" t="inlineStr">
-        <is>
-          <t>W1</t>
-        </is>
-      </c>
-      <c r="B11" s="33" t="inlineStr">
-        <is>
-          <t>06 Jul</t>
-        </is>
-      </c>
-      <c r="C11" s="33" t="inlineStr">
-        <is>
-          <t>Dashboard core widgets live (AI card → R34)</t>
-        </is>
-      </c>
-      <c r="D11" s="34" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E11" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F11" s="33" t="inlineStr">
+      <c r="J22" s="45" t="inlineStr">
+        <is>
+          <t>⬆ 100% on 2026-07-23 — the composite methodology is now real. The fear-greed.job computes the true 4-component composite (momentum from SPY vs its 125-day MA, safe-haven from SPY−TLT 20-day return spread, volatility from VIXY vs its 50-day MA, breadth from grouped-daily advancers) for both the live value and a backfilled market_sentiment_history/{date} series (25 trading days, verified). The dashboard sparkline now reads that real composite history instead of the breadth-only proxy. The earlier missing-rule bug (gauge silently rendering a hardcoded 62) was fixed on 07-22; market_sentiment_history rule added and released 07-23.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="46" t="inlineStr">
+        <is>
+          <t>R28</t>
+        </is>
+      </c>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C23" s="46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D23" s="47" t="inlineStr">
+        <is>
+          <t>Recaps EOD data job</t>
+        </is>
+      </c>
+      <c r="E23" s="47" t="inlineStr">
+        <is>
+          <t>Polygon (composed)</t>
+        </is>
+      </c>
+      <c r="F23" s="47" t="inlineStr">
+        <is>
+          <t>Composes market_indices / market_movers / sectors / market_breadth → recaps/{date}</t>
+        </is>
+      </c>
+      <c r="G23" s="47" t="inlineStr">
+        <is>
+          <t>Recap · end-of-day recap</t>
+        </is>
+      </c>
+      <c r="H23" s="46" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I23" s="47" t="inlineStr">
+        <is>
+          <t>AI prose lead + news briefing → R36 (Anthropic), separately tracked</t>
+        </is>
+      </c>
+      <c r="J23" s="47" t="inlineStr">
+        <is>
+          <t>⬆ 0% → 100% on 2026-07-23. New recaps.job (cron 45 18 * * 1-5, Scheduler sync-recaps registered) freezes each session's indices, top gainers/losers, sector leaders/laggards and market internals (advancers/decliners/breadth/TRIN/up-down volume) into one dated snapshot — Polygon-derived, no extra vendor call. recap.tsx now renders the live recaps/{date} doc: hero index tiles, Biggest Movers, Market Internals and the drawer A/D bar are real; the fabricated 'extended breadth' block (NYSE TICK / McClellan / Put-Call — not available from Polygon) was deleted. Verified: recaps/2026-07-21 written with 9 indices, 6+6 movers, 3+3 sectors, real internals. The prose lead + news briefing remain AI narrative → R36 (Anthropic, your planned purchase), the only recap sub-part not part of this data-job row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="44" t="inlineStr">
+        <is>
+          <t>R29</t>
+        </is>
+      </c>
+      <c r="B24" s="44" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C24" s="44" t="inlineStr">
+        <is>
+          <t>🔵→</t>
+        </is>
+      </c>
+      <c r="D24" s="45" t="inlineStr">
+        <is>
+          <t>10-quarter EPS history (quarterly financials + wire)</t>
+        </is>
+      </c>
+      <c r="E24" s="45" t="inlineStr">
+        <is>
+          <t>Polygon (actuals) — estimates need Benzinga add-on</t>
+        </is>
+      </c>
+      <c r="F24" s="45" t="inlineStr">
+        <is>
+          <t>Polygon /vX/reference/financials (actuals). Estimate feed: Polygon Benzinga Earnings add-on (not on current plan)</t>
+        </is>
+      </c>
+      <c r="G24" s="45" t="inlineStr">
+        <is>
+          <t>Earnings hub · EPS &amp; Sales / Income statement</t>
+        </is>
+      </c>
+      <c r="H24" s="44" t="inlineStr">
+        <is>
+          <t>90% ⬇</t>
+        </is>
+      </c>
+      <c r="I24" s="45" t="inlineStr">
+        <is>
+          <t>EPS estimates — the forward/estimate side has no redistributable source on the current plan. FMP/Finnhub estimates exist in code but are NOT licensed for redistribution, so they must not ship to users</t>
+        </is>
+      </c>
+      <c r="J24" s="45" t="inlineStr">
+        <is>
+          <t>⬇ Recapped from 98% → 90% on 2026-07-23 to reflect the redistribution constraint honestly. The actuals are 100% Polygon and redistributable: 10 real quarters of EPS from /vX/reference/financials (~228 tickers), plus full balance sheet, cash flow, margins and current ratio — a complete fundamentals panel. The estimate overlay (actual-vs-estimate beat/miss) is the only gap: the only sources wired are FMP/Finnhub, which are not redistributable, so per the Polygon-only policy they cannot be served. A redistribution-legal estimate feed = Polygon's Benzinga Earnings &amp; Estimates add-on (a paid add-on to the current plan, tracked with R41/R42). Until purchased, estimates stay unshipped and this row is capped below 100%. ⬆ 2026-07-24 — actuals scope widened again (row still 90%, gap unchanged): financials now also carry 8 annual fiscal years (income/balance/cash-flow via timeframe=annual), so the earnings hub gained Quarterly / Yearly tabs on both EPS &amp; Sales history and the Income statement (actuals only, chart removed). The 90% cap is unmoved because it reflects the missing *estimate* feed, not the actuals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="46" t="inlineStr">
+        <is>
+          <t>R30</t>
+        </is>
+      </c>
+      <c r="B25" s="46" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C25" s="46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D25" s="47" t="inlineStr">
+        <is>
+          <t>Screener sector/cap class + IPO recent perf + Macro regime label</t>
+        </is>
+      </c>
+      <c r="E25" s="47" t="inlineStr">
+        <is>
+          <t>Polygon</t>
+        </is>
+      </c>
+      <c r="F25" s="47" t="inlineStr">
+        <is>
+          <t>/v3/reference/tickers (class) + market_indices/market_breadth (regime)</t>
+        </is>
+      </c>
+      <c r="G25" s="47" t="inlineStr">
+        <is>
+          <t>Screener / IPOs / Macro · sector-cap class, IPO perf, regime label</t>
+        </is>
+      </c>
+      <c r="H25" s="46" t="inlineStr">
+        <is>
+          <t>100% ✅</t>
+        </is>
+      </c>
+      <c r="I25" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="33" t="inlineStr">
-        <is>
-          <t>W2</t>
-        </is>
-      </c>
-      <c r="B12" s="33" t="inlineStr">
-        <is>
-          <t>13 Jul</t>
-        </is>
-      </c>
-      <c r="C12" s="33" t="inlineStr">
-        <is>
-          <t>Macro &amp; VIX live (econ calendar + dividends + VIX/yields)</t>
-        </is>
-      </c>
-      <c r="D12" s="35" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E12" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F12" s="33" t="inlineStr">
+      <c r="J25" s="47" t="inlineStr">
+        <is>
+          <t>⬆ 70% → 100% on 2026-07-23 — all 3 sub-parts done. ✅ Sector/cap classification live (companies). ✅ IPO aftermarket perf live (ipos.job, Polygon /v2/aggs). ✅ Macro regime label now computed: macro.tsx derives Risk-On / Neutral / Risk-Off by voting three live signals — VIX/VIXY level, market breadth (adv/dec from market_breadth) and the 10-year Treasury yield — replacing the hardcoded 'Risk-On Rally'. All Polygon/public data, no vendor purchase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="44" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B26" s="44" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="C26" s="44" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D26" s="45" t="inlineStr">
+        <is>
+          <t>Options Chain live (bid/ask/IV/OI/Greeks)</t>
+        </is>
+      </c>
+      <c r="E26" s="45" t="inlineStr">
+        <is>
+          <t>Polygon → Tradier</t>
+        </is>
+      </c>
+      <c r="F26" s="45" t="inlineStr">
+        <is>
+          <t>Polygon /v3/reference/options/contracts + /v2/aggs/ticker/O:{contract}/range/1/day/…; Tradier /v1/markets/options/chains (quotes — 🔴 unwired). Polygon /v3/snapshot/options → 403</t>
+        </is>
+      </c>
+      <c r="G26" s="45" t="inlineStr">
+        <is>
+          <t>Options · options chain</t>
+        </is>
+      </c>
+      <c r="H26" s="44" t="inlineStr">
+        <is>
+          <t>45% ⬆</t>
+        </is>
+      </c>
+      <c r="I26" s="45" t="inlineStr">
+        <is>
+          <t>Greeks, IV, open interest and bid/ask are still 🔴 hard-blocked — Polygon's options *snapshot* endpoint returns NOT_AUTHORIZED on the current plan (re-probed live 2026-07-22, still 403). Those four columns cannot be made real without a vendor purchase</t>
+        </is>
+      </c>
+      <c r="J26" s="45" t="inlineStr">
+        <is>
+          <t>⬆ Raised from 25%, but read the nuance — the block has NOT lifted. What changed is a different endpoint: option contract aggregates *are* authorized, so options-chains.job.ts now writes real per-contract OHLC, VWAP, trade count and range %. So the chain is no longer wholly synthetic — traded price/volume history per contract is genuine market data. But the quote-side surface a user actually reads an options chain for (bid/ask spread, IV, OI, greeks) is still fabricated. Unblock = Tradier (token already held, unwired) or Polygon Options Advanced</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="46" t="inlineStr">
+        <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B27" s="46" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="C27" s="46" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D27" s="47" t="inlineStr">
+        <is>
+          <t>ENABLER: AI service + ANTHROPIC key + prompt infra</t>
+        </is>
+      </c>
+      <c r="E27" s="47" t="inlineStr">
+        <is>
+          <t>Anthropic (deferred)</t>
+        </is>
+      </c>
+      <c r="F27" s="47" t="inlineStr">
+        <is>
+          <t>— (unwired by decision)</t>
+        </is>
+      </c>
+      <c r="G27" s="47" t="inlineStr">
+        <is>
+          <t>— *(AI enabler)*</t>
+        </is>
+      </c>
+      <c r="H27" s="46" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I27" s="47" t="inlineStr">
+        <is>
+          <t>AI service</t>
+        </is>
+      </c>
+      <c r="J27" s="47" t="inlineStr">
+        <is>
+          <t>⏸️ Deferred by decision (2026-07-21) — you chose labeled placeholders over wiring Anthropic this phase. Not blocked: ANTHROPIC_API_KEY is provisioned; this is a scope choice to avoid per-request LLM cost until later</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="44" t="inlineStr">
+        <is>
+          <t>R35</t>
+        </is>
+      </c>
+      <c r="B28" s="44" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="C28" s="44" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D28" s="45" t="inlineStr">
+        <is>
+          <t>Dashboard 'What Matters Now' AI card</t>
+        </is>
+      </c>
+      <c r="E28" s="45" t="inlineStr">
+        <is>
+          <t>Anthropic (deferred)</t>
+        </is>
+      </c>
+      <c r="F28" s="45" t="inlineStr">
+        <is>
+          <t>— (unwired by decision)</t>
+        </is>
+      </c>
+      <c r="G28" s="45" t="inlineStr">
+        <is>
+          <t>Dashboard · "What Matters Now" (AI — unwired)</t>
+        </is>
+      </c>
+      <c r="H28" s="44" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I28" s="45" t="inlineStr">
+        <is>
+          <t>Real AI narrative</t>
+        </is>
+      </c>
+      <c r="J28" s="45" t="inlineStr">
+        <is>
+          <t>⏸️ Deferred by decision — card ships as a labeled placeholder; becomes real once R34 (Anthropic) is switched on</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="46" t="inlineStr">
+        <is>
+          <t>R36</t>
+        </is>
+      </c>
+      <c r="B29" s="46" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="C29" s="46" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D29" s="47" t="inlineStr">
+        <is>
+          <t>Recaps AI narrative</t>
+        </is>
+      </c>
+      <c r="E29" s="47" t="inlineStr">
+        <is>
+          <t>Anthropic (deferred)</t>
+        </is>
+      </c>
+      <c r="F29" s="47" t="inlineStr">
+        <is>
+          <t>— (unwired by decision)</t>
+        </is>
+      </c>
+      <c r="G29" s="47" t="inlineStr">
+        <is>
+          <t>Recap · AI narrative (unwired)</t>
+        </is>
+      </c>
+      <c r="H29" s="46" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I29" s="47" t="inlineStr">
+        <is>
+          <t>Real AI narrative</t>
+        </is>
+      </c>
+      <c r="J29" s="47" t="inlineStr">
+        <is>
+          <t>⏸️ Deferred by decision (AI) + depends on R28 recap job (Milestone 3, in progress). Data layer will exist; only the LLM narrative is held back</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="44" t="inlineStr">
+        <is>
+          <t>R38</t>
+        </is>
+      </c>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="C30" s="44" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D30" s="45" t="inlineStr">
+        <is>
+          <t>Stock Detail AI (thesis/risk/confidence + technical analysis)</t>
+        </is>
+      </c>
+      <c r="E30" s="45" t="inlineStr">
+        <is>
+          <t>Anthropic (deferred)</t>
+        </is>
+      </c>
+      <c r="F30" s="45" t="inlineStr">
+        <is>
+          <t>— (unwired by decision)</t>
+        </is>
+      </c>
+      <c r="G30" s="45" t="inlineStr">
+        <is>
+          <t>Stock detail · AI thesis / risk (unwired)</t>
+        </is>
+      </c>
+      <c r="H30" s="44" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I30" s="45" t="inlineStr">
+        <is>
+          <t>Real AI</t>
+        </is>
+      </c>
+      <c r="J30" s="45" t="inlineStr">
+        <is>
+          <t>⏸️ Deferred by decision — template text is honestly labeled 'AI-generated'; real model output awaits R34</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="46" t="inlineStr">
+        <is>
+          <t>R39</t>
+        </is>
+      </c>
+      <c r="B31" s="46" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="C31" s="46" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D31" s="47" t="inlineStr">
+        <is>
+          <t>Earnings+Analyst+Insider+Watchlist AI notes</t>
+        </is>
+      </c>
+      <c r="E31" s="47" t="inlineStr">
+        <is>
+          <t>Anthropic (deferred)</t>
+        </is>
+      </c>
+      <c r="F31" s="47" t="inlineStr">
+        <is>
+          <t>— (unwired by decision)</t>
+        </is>
+      </c>
+      <c r="G31" s="47" t="inlineStr">
+        <is>
+          <t>Earnings / Analyst / Insider / Watchlist · AI notes (unwired)</t>
+        </is>
+      </c>
+      <c r="H31" s="46" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I31" s="47" t="inlineStr">
+        <is>
+          <t>Real AI</t>
+        </is>
+      </c>
+      <c r="J31" s="47" t="inlineStr">
+        <is>
+          <t>⏸️ Deferred by decision (AI). Includes R20 watchlist AI summary — non-AI watchlist parts already at 100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="44" t="inlineStr">
+        <is>
+          <t>R41</t>
+        </is>
+      </c>
+      <c r="B32" s="44" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="C32" s="44" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D32" s="45" t="inlineStr">
+        <is>
+          <t>Analyst Actions per-firm event table (upgrades/downgrades/PT)</t>
+        </is>
+      </c>
+      <c r="E32" s="45" t="inlineStr">
+        <is>
+          <t>Benzinga (🔴 403) / FMP</t>
+        </is>
+      </c>
+      <c r="F32" s="45" t="inlineStr">
+        <is>
+          <t>Benzinga /benzinga/v1/ratings → 403; FMP grades-consensus (snapshot only)</t>
+        </is>
+      </c>
+      <c r="G32" s="45" t="inlineStr">
+        <is>
+          <t>Analyst · per-firm event table</t>
+        </is>
+      </c>
+      <c r="H32" s="44" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="I32" s="45" t="inlineStr">
+        <is>
+          <t>Per-firm upgrade/downgrade events</t>
+        </is>
+      </c>
+      <c r="J32" s="45" t="inlineStr">
+        <is>
+          <t>🔴 Vendor-blocked, not effort — per-firm actions need Benzinga (403 on current plan). FMP gives only a consensus snapshot; Finnhub gives rating *history* but not per-firm. Requires a paid vendor decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="46" t="inlineStr">
+        <is>
+          <t>R42</t>
+        </is>
+      </c>
+      <c r="B33" s="46" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="C33" s="46" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="inlineStr">
+        <is>
+          <t>Earnings depth (guidance/reaction/real-time actuals + tags)</t>
+        </is>
+      </c>
+      <c r="E33" s="47" t="inlineStr">
+        <is>
+          <t>FMP + Benzinga (🔴 403)</t>
+        </is>
+      </c>
+      <c r="F33" s="47" t="inlineStr">
+        <is>
+          <t>FMP /stable/earnings-calendar; Benzinga /benzinga/v1/{earnings,guidance} → 403; reaction derivable from ohlcv_bars</t>
+        </is>
+      </c>
+      <c r="G33" s="47" t="inlineStr">
+        <is>
+          <t>Earnings hub · guidance / reaction depth</t>
+        </is>
+      </c>
+      <c r="H33" s="46" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="I33" s="47" t="inlineStr">
+        <is>
+          <t>Guidance + price reaction</t>
+        </is>
+      </c>
+      <c r="J33" s="47" t="inlineStr">
+        <is>
+          <t>🟠 Partially unblockable now — session (BMO/AMC) IS available on the held Finnhub key (unwired); guidance/reaction still need a Benzinga-class feed. Reaction could also be computed from ohlcv_bars post-print</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="44" t="inlineStr">
+        <is>
+          <t>R43</t>
+        </is>
+      </c>
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="C34" s="44" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D34" s="45" t="inlineStr">
+        <is>
+          <t>Options flow + dark-pool prints</t>
+        </is>
+      </c>
+      <c r="E34" s="45" t="inlineStr">
+        <is>
+          <t>Unusual Whales (not subscribed)</t>
+        </is>
+      </c>
+      <c r="F34" s="45" t="inlineStr">
+        <is>
+          <t>— (unwired)</t>
+        </is>
+      </c>
+      <c r="G34" s="45" t="inlineStr">
+        <is>
+          <t>Options · flow + dark-pool prints</t>
+        </is>
+      </c>
+      <c r="H34" s="44" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I34" s="45" t="inlineStr">
+        <is>
+          <t>Entire feature</t>
+        </is>
+      </c>
+      <c r="J34" s="45" t="inlineStr">
+        <is>
+          <t>🔴 Vendor-blocked — needs a UnusualWhales / Polygon-paid flow add-on the current plans don't include. Marked P2 (post-MVP) in the plan itself</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="46" t="inlineStr">
+        <is>
+          <t>R44</t>
+        </is>
+      </c>
+      <c r="B35" s="46" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="C35" s="46" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D35" s="47" t="inlineStr">
+        <is>
+          <t>Alerts engine (12 alert types + watchlist toggles)</t>
+        </is>
+      </c>
+      <c r="E35" s="47" t="inlineStr">
+        <is>
+          <t>— (internal)</t>
+        </is>
+      </c>
+      <c r="F35" s="47" t="inlineStr">
+        <is>
+          <t>— (rules over synced Firestore data)</t>
+        </is>
+      </c>
+      <c r="G35" s="47" t="inlineStr">
+        <is>
+          <t>Alerts · alerts engine (screen not built)</t>
+        </is>
+      </c>
+      <c r="H35" s="46" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="I35" s="47" t="inlineStr">
+        <is>
+          <t>Rules engine + 12 alert types</t>
+        </is>
+      </c>
+      <c r="J35" s="47" t="inlineStr">
+        <is>
+          <t>🔨 Not built — no blocker. Net-new backend (evaluate rules against synced data, per-user toggles, delivery). All input data exists; it is buildable now, just not yet scheduled (W9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="44" t="inlineStr">
+        <is>
+          <t>R46</t>
+        </is>
+      </c>
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="C36" s="44" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D36" s="45" t="inlineStr">
+        <is>
+          <t>Editorial + dropped-feature decisions</t>
+        </is>
+      </c>
+      <c r="E36" s="45" t="inlineStr">
+        <is>
+          <t>— (product)</t>
+        </is>
+      </c>
+      <c r="F36" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>W2</t>
-        </is>
-      </c>
-      <c r="B13" s="33" t="inlineStr">
-        <is>
-          <t>13 Jul</t>
-        </is>
-      </c>
-      <c r="C13" s="33" t="inlineStr">
-        <is>
-          <t>IPOs live (calendar + offer price)</t>
-        </is>
-      </c>
-      <c r="D13" s="35" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E13" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F13" s="33" t="inlineStr">
+      <c r="G36" s="45" t="inlineStr">
+        <is>
+          <t>— *(product decisions)*</t>
+        </is>
+      </c>
+      <c r="H36" s="44" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I36" s="45" t="inlineStr">
+        <is>
+          <t>Product decisions</t>
+        </is>
+      </c>
+      <c r="J36" s="45" t="inlineStr">
+        <is>
+          <t>🗓️ W10 by design — a decision/curation task (which themes, presets, sections to keep or cut), correctly sequenced for launch week; not an engineering gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="46" t="inlineStr">
+        <is>
+          <t>R47</t>
+        </is>
+      </c>
+      <c r="B37" s="46" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="C37" s="46" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D37" s="47" t="inlineStr">
+        <is>
+          <t>Earnings + Macro calendars on real date ranges (structural)</t>
+        </is>
+      </c>
+      <c r="E37" s="47" t="inlineStr">
+        <is>
+          <t>FMP + Finnhub</t>
+        </is>
+      </c>
+      <c r="F37" s="47" t="inlineStr">
+        <is>
+          <t>FMP /stable/earnings-calendar; Finnhub /calendar/economic</t>
+        </is>
+      </c>
+      <c r="G37" s="47" t="inlineStr">
+        <is>
+          <t>Earnings + Macro calendars · date-anchored calendars</t>
+        </is>
+      </c>
+      <c r="H37" s="46" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
+      <c r="I37" s="47" t="inlineStr">
+        <is>
+          <t>Earnings coverage thin</t>
+        </is>
+      </c>
+      <c r="J37" s="47" t="inlineStr">
+        <is>
+          <t>Ahead of schedule — date-anchored calendar built (earnings-calendar.tsx, calendar-range.ts); FMP's 10-row coverage limits it</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="44" t="inlineStr">
+        <is>
+          <t>R48</t>
+        </is>
+      </c>
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="C38" s="44" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D38" s="45" t="inlineStr">
+        <is>
+          <t>Full regression + empty-states + mobile + performance</t>
+        </is>
+      </c>
+      <c r="E38" s="45" t="inlineStr">
+        <is>
+          <t>— (QA)</t>
+        </is>
+      </c>
+      <c r="F38" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G13" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="33" t="inlineStr">
-        <is>
-          <t>W2</t>
-        </is>
-      </c>
-      <c r="B14" s="33" t="inlineStr">
-        <is>
-          <t>13 Jul</t>
-        </is>
-      </c>
-      <c r="C14" s="33" t="inlineStr">
-        <is>
-          <t>Commentary/News live (aggregated feed + tags + drawer)</t>
-        </is>
-      </c>
-      <c r="D14" s="34" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E14" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F14" s="33" t="inlineStr">
+      <c r="G38" s="45" t="inlineStr">
+        <is>
+          <t>— *(QA)*</t>
+        </is>
+      </c>
+      <c r="H38" s="44" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I38" s="45" t="inlineStr">
+        <is>
+          <t>QA gate</t>
+        </is>
+      </c>
+      <c r="J38" s="45" t="inlineStr">
+        <is>
+          <t>🗓️ W10 by design — final QA/regression gate, only meaningful once features stop changing. Partially advanced by R21 empty-state work</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="46" t="inlineStr">
+        <is>
+          <t>R49</t>
+        </is>
+      </c>
+      <c r="B39" s="46" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="C39" s="46" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="D39" s="47" t="inlineStr">
+        <is>
+          <t>Security review + launch checklist</t>
+        </is>
+      </c>
+      <c r="E39" s="47" t="inlineStr">
+        <is>
+          <t>— (security)</t>
+        </is>
+      </c>
+      <c r="F39" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G14" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="33" t="inlineStr">
-        <is>
-          <t>W2</t>
-        </is>
-      </c>
-      <c r="B15" s="33" t="inlineStr">
-        <is>
-          <t>13 Jul</t>
-        </is>
-      </c>
-      <c r="C15" s="33" t="inlineStr">
-        <is>
-          <t>Sector Themes live (per-stock prices + theme perf)</t>
-        </is>
-      </c>
-      <c r="D15" s="34" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E15" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F15" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>W2</t>
-        </is>
-      </c>
-      <c r="B16" s="33" t="inlineStr">
-        <is>
-          <t>13 Jul</t>
-        </is>
-      </c>
-      <c r="C16" s="33" t="inlineStr">
-        <is>
-          <t>Company-name search (nameLower/tokens)</t>
-        </is>
-      </c>
-      <c r="D16" s="35" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E16" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app</t>
-        </is>
-      </c>
-      <c r="F16" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="33" t="inlineStr">
-        <is>
-          <t>Complete — ALL search boxes now match ticker AND company name over the live universe: ⌘K palette, the Search page (was ticker-only), and the Watchlist/Portfolio add modals (new live typeahead). Options/Commentary already matched name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
-      </c>
-      <c r="B17" s="33" t="inlineStr">
-        <is>
-          <t>20 Jul</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="inlineStr">
-        <is>
-          <t>Portfolio Pulse live (holdings + prices + P&amp;L + totals)</t>
-        </is>
-      </c>
-      <c r="D17" s="34" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E17" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F17" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="33" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
-      </c>
-      <c r="B18" s="33" t="inlineStr">
-        <is>
-          <t>20 Jul</t>
-        </is>
-      </c>
-      <c r="C18" s="33" t="inlineStr">
-        <is>
-          <t>Watchlist live (persistence + prices + AI summary)</t>
-        </is>
-      </c>
-      <c r="D18" s="34" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E18" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F18" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="33" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
-      </c>
-      <c r="B19" s="33" t="inlineStr">
-        <is>
-          <t>20 Jul</t>
-        </is>
-      </c>
-      <c r="C19" s="33" t="inlineStr">
-        <is>
-          <t>Empty-states + graceful fallback polish (cross-screen)</t>
-        </is>
-      </c>
-      <c r="D19" s="34" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E19" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F19" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="38" t="inlineStr">
-        <is>
-          <t>— Milestone 1 &amp; 2 items (W4/W5), delivered early this session —</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="33" t="inlineStr">
-        <is>
-          <t>W4</t>
-        </is>
-      </c>
-      <c r="B21" s="33" t="inlineStr">
-        <is>
-          <t>27 Jul</t>
-        </is>
-      </c>
-      <c r="C21" s="33" t="inlineStr">
-        <is>
-          <t>Stock Detail live — financials/EPS/pivots (Milestone 1)</t>
-        </is>
-      </c>
-      <c r="D21" s="34" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E21" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F21" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="33" t="inlineStr">
-        <is>
-          <t>W4</t>
-        </is>
-      </c>
-      <c r="B22" s="33" t="inlineStr">
-        <is>
-          <t>27 Jul</t>
-        </is>
-      </c>
-      <c r="C22" s="33" t="inlineStr">
-        <is>
-          <t>Dashboard Fear &amp; Greed gauge live (Milestone 2)</t>
-        </is>
-      </c>
-      <c r="D22" s="35" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E22" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F22" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="33" t="inlineStr">
-        <is>
-          <t>Complete — verified live; see DELIVERY-PLAN-STATUS.md (2026-07-24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="33" t="inlineStr">
-        <is>
-          <t>W5</t>
-        </is>
-      </c>
-      <c r="B23" s="33" t="inlineStr">
-        <is>
-          <t>03 Aug</t>
-        </is>
-      </c>
-      <c r="C23" s="33" t="inlineStr">
-        <is>
-          <t>10-quarter EPS history (Milestone 1)</t>
-        </is>
-      </c>
-      <c r="D23" s="35" t="inlineStr">
-        <is>
-          <t>90%</t>
-        </is>
-      </c>
-      <c r="E23" s="33" t="inlineStr">
-        <is>
-          <t>✅ Deployed — UI marketcatalyst.web.app + backend Cloud Run rev 00023</t>
-        </is>
-      </c>
-      <c r="F23" s="33" t="inlineStr">
-        <is>
-          <t>Estimate overlay (actual-vs-estimate beat/miss) has no redistributable source on Polygon Stocks Starter. The 10 quarters of EPS ACTUALS are 100% and now also drive Quarterly/Yearly EPS &amp; Sales + Income-statement tabs (8 annual years added 2026-07-24).</t>
-        </is>
-      </c>
-      <c r="G23" s="33" t="inlineStr">
-        <is>
-          <t>Purchase Polygon's Benzinga Earnings &amp; Estimates add-on to ship forward EPS + %-surprise. Cannot reach 100% on current data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="39" t="inlineStr">
-        <is>
-          <t>ROLLUP</t>
-        </is>
-      </c>
-      <c r="C25" s="40" t="inlineStr">
-        <is>
-          <t>18 deliverables · avg ~99% · 17 at 100% · 1 at 90% (10-qtr EPS — estimate overlay needs Benzinga)</t>
+      <c r="G39" s="47" t="inlineStr">
+        <is>
+          <t>— *(security)*</t>
+        </is>
+      </c>
+      <c r="H39" s="46" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="I39" s="47" t="inlineStr">
+        <is>
+          <t>Full review + checklist</t>
+        </is>
+      </c>
+      <c r="J39" s="47" t="inlineStr">
+        <is>
+          <t>🗓️ W10 by design. Already done ahead: runtime SA least-privilege; Firestore rules server-write-only; retention module; 2026-07-22 rules hardening — plans writable by admin on featureFlags+updatedAt only (a client that could rewrite amount could set a plan to $0), create/delete denied; feature_adoption is the only client-writable analytics collection and is constrained (row must belong to caller, openCount may only increase, ownership immutable, delete denied); adminDashboard/userManagement are staff-only on every plan so they can never be sold (privilege escalation). ⚠️ Still outstanding, all three real: (1) POLYGON_API_KEY is still un-rotated (exposed in chat; Secret Manager version 4 enabled; deploy/rotate-polygon-key.sh automates all of it except generating the replacement). (2) ✅ Resolved 2026-07-23 without the risky rewrite. Backend reachability was delivered by a SEPARATE public service (market-catalyst-live, APP_ROLE=live) that mounts only LiveModule — /sync, /purge, /retention, /admin all return 404 there (verified) while the worker stays --no-allow-unauthenticated with ADMIN_GUARD_TRUST_IAM=true. No Hosting→Cloud Run rewrite was used, so the world-callable-admin risk never materialised. (3) Both repos ship a firestore.rules and they have drifted — the live ruleset deploys from MarketCatalystUI/firestore.rules; the backend copy is stale and now carries a DO-NOT-DEPLOY header</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
after removing static data
</commit_message>
<xml_diff>
--- a/Doc/MarketCatalyst.ai_weekly_deliverables_Plan.xlsx
+++ b/Doc/MarketCatalyst.ai_weekly_deliverables_Plan.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Row-by-Row Status" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Plan (W1-W10)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Path to 100%" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -131,7 +132,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -213,6 +214,26 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2DCDB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -269,7 +290,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -378,6 +399,31 @@
     <xf numFmtId="0" fontId="19" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -768,1929 +814,1929 @@
     <row r="2" ht="30" customHeight="1" s="27">
       <c r="A2" s="42" t="inlineStr">
         <is>
-          <t>State sync 2026-07-24 · all 36 rows · Polygon/Massive is the only vendor served to users. 'Screen · Feature' = the app screen this row powers (— for infra/enabler/AI-unwired rows).</t>
+          <t>State sync 2026-07-29 · all 36 rows, corrected · exact copy of DELIVERY-PLAN-STATUS.md, refreshed from the 2026-07-24 snapshot to fold in the 2026-07-26 on-demand-architecture redesign, the 2026-07-27 two-environment (stage+prod) rollout, and the 2026-07-29 evidence-correction pass. Row % values are unchanged from 2026-07-24 — only stale mechanism citations were corrected (see ⚠️/❓ markers inline) and two rows (R16, R25) were flagged as needing live re-verification rather than reasserted.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1" s="27">
-      <c r="A3" s="43" t="inlineStr">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>Row</t>
         </is>
       </c>
-      <c r="B3" s="43" t="inlineStr">
+      <c r="B3" s="48" t="inlineStr">
         <is>
           <t>Wk</t>
         </is>
       </c>
-      <c r="C3" s="43" t="inlineStr">
+      <c r="C3" s="48" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="D3" s="43" t="inlineStr">
+      <c r="D3" s="48" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
       </c>
-      <c r="E3" s="43" t="inlineStr">
+      <c r="E3" s="48" t="inlineStr">
         <is>
           <t>Provider</t>
         </is>
       </c>
-      <c r="F3" s="43" t="inlineStr">
+      <c r="F3" s="48" t="inlineStr">
         <is>
           <t>API URL</t>
         </is>
       </c>
-      <c r="G3" s="43" t="inlineStr">
+      <c r="G3" s="48" t="inlineStr">
         <is>
           <t>Screen · Feature</t>
         </is>
       </c>
-      <c r="H3" s="43" t="inlineStr">
+      <c r="H3" s="48" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="I3" s="43" t="inlineStr">
+      <c r="I3" s="48" t="inlineStr">
         <is>
           <t>What's NOT done</t>
         </is>
       </c>
-      <c r="J3" s="43" t="inlineStr">
+      <c r="J3" s="48" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="49" t="inlineStr">
         <is>
           <t>R5</t>
         </is>
       </c>
-      <c r="B4" s="44" t="inlineStr">
+      <c r="B4" s="49" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="C4" s="44" t="inlineStr">
+      <c r="C4" s="49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D4" s="45" t="inlineStr">
+      <c r="D4" s="49" t="inlineStr">
         <is>
           <t>FOUNDATION: deploy FE+BE 24/7, Blaze, service-account, indexes+TTL</t>
         </is>
       </c>
-      <c r="E4" s="45" t="inlineStr">
+      <c r="E4" s="49" t="inlineStr">
         <is>
           <t>Firebase / Cloud Run</t>
         </is>
       </c>
-      <c r="F4" s="45" t="inlineStr">
+      <c r="F4" s="49" t="inlineStr">
         <is>
           <t>— (infra: Hosting + Cloud Run + Firestore)</t>
         </is>
       </c>
-      <c r="G4" s="45" t="inlineStr">
-        <is>
-          <t>— *(infra)*</t>
-        </is>
-      </c>
-      <c r="H4" s="44" t="inlineStr">
+      <c r="G4" s="49" t="inlineStr">
+        <is>
+          <t>— (infra)</t>
+        </is>
+      </c>
+      <c r="H4" s="49" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I4" s="45" t="inlineStr">
+      <c r="I4" s="49" t="inlineStr">
         <is>
           <t>— (R5 scope fully delivered; the Polygon key rotation + rules-drift items are R49's scope, separately tracked — not a dependency of this row)</t>
         </is>
       </c>
-      <c r="J4" s="45" t="inlineStr">
-        <is>
-          <t>✅ Complete 2026-07-23. Every element of R5's stated scope is delivered and verified: deploy FE+BE (FE marketcatalyst.web.app; worker rev 00035-d74 + public market-catalyst-live), 24/7 (21 Cloud Scheduler jobs ENABLED and firing on schedule — sync-companies 2026-07-23 06:00 UTC, sync-news 20:30 UTC, sync-market-movers 22:00 UTC — all matching their crons; scheduler-invoker SA present), Blaze (Cloud Run + Scheduler operating), service-account (runtime SA least-privilege: datastore.user+secretAccessor), indexes (deployed), TTL (not possible on ISO-string dates → substituted with the in-code retention module, weekly prune, RETENTION_DRY_RUN=false). Backend is browser-reachable and CORS-verified. Security follow-ups live in R49, not here.</t>
+      <c r="J4" s="49" t="inlineStr">
+        <is>
+          <t>✅ Complete 2026-07-23. Every element of R5's stated scope is delivered and verified: deploy FE+BE (FE marketcatalyst.web.app; worker rev 00035-d74 + public market-catalyst-live), 24/7 (21 Cloud Scheduler jobs ENABLED and firing on schedule — sync-companies 2026-07-23 06:00 UTC, sync-news 20:30 UTC, sync-market-movers 22:00 UTC — all matching their crons; scheduler-invoker SA present), Blaze (Cloud Run + Scheduler operating), service-account (runtime SA least-privilege: datastore.user+secretAccessor), indexes (deployed), TTL (not possible on ISO-string dates → substituted with the in-code retention module, weekly prune, RETENTION_DRY_RUN=false). Backend is browser-reachable and CORS-verified. Security follow-ups live in R49, not here. ⚠️ 2026-07-29: the 21-job evidence above predates the 2026-07-26 redesign — those jobs were deleted and replaced by a single sync-premarket cron; "24/7" is now delivered by the always-on public live Cloud Run service + on-demand TTL-based freshness, not scheduled-job cadence. Row stays 100% (the deliverable — FE+BE always reachable — is if anything stronger now), but the cited mechanism is obsolete. Not independently re-verified against live production this pass (gcloud session in this environment needs interactive re-auth).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="46" t="inlineStr">
+      <c r="A5" s="50" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
-      <c r="B5" s="46" t="inlineStr">
+      <c r="B5" s="50" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="C5" s="46" t="inlineStr">
+      <c r="C5" s="50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D5" s="47" t="inlineStr">
+      <c r="D5" s="50" t="inlineStr">
         <is>
           <t>Feature-flag system (feature_flags doc, per-release FF_* toggles)</t>
         </is>
       </c>
-      <c r="E5" s="47" t="inlineStr">
+      <c r="E5" s="50" t="inlineStr">
         <is>
           <t>— (internal)</t>
         </is>
       </c>
-      <c r="F5" s="47" t="inlineStr">
+      <c r="F5" s="50" t="inlineStr">
         <is>
           <t>— (Firestore feature_flags)</t>
         </is>
       </c>
-      <c r="G5" s="47" t="inlineStr">
-        <is>
-          <t>— *(internal)*</t>
-        </is>
-      </c>
-      <c r="H5" s="46" t="inlineStr">
+      <c r="G5" s="50" t="inlineStr">
+        <is>
+          <t>— (internal)</t>
+        </is>
+      </c>
+      <c r="H5" s="50" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="I5" s="47" t="inlineStr">
+      <c r="I5" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J5" s="47" t="inlineStr">
-        <is>
-          <t>Built 2026-07-21: registry + service + API + UI provider/Gate + nav &amp; screen gating. Deployed rev 00017; feature_flags/default auto-seeded 25 flags in prod; resolver verified (default→env→Firestore, fail-open). Extended 2026-07-22 with a SECOND, independent gating layer — per-plan entitlements (src/plans/plans.registry.ts, 16 keys × 3 plans) plus an admin UI to edit them per plan (public/admin/console.html feature editor, writing plans/{id}.featureFlags under a rules constraint that permits only featureFlags+updatedAt). The two layers are deliberately NOT merged: FF_* answers *"is it built and shipped?"* → "coming soon"; entitlements answer *"may this tier use it?"* → "upgrade to unlock". Merging them would make an unbuilt feature masquerade as a paywall. Scope exceeded, not just met</t>
+      <c r="J5" s="50" t="inlineStr">
+        <is>
+          <t>Built 2026-07-21: registry + service + API + UI provider/Gate + nav &amp; screen gating. Deployed rev 00017; feature_flags/default auto-seeded 25 flags in prod; resolver verified (default→env→Firestore, fail-open). Extended 2026-07-22 with a SECOND, independent gating layer — per-plan entitlements (src/plans/plans.registry.ts, 16 keys × 3 plans) plus an admin UI to edit them per plan (public/admin/console.html feature editor, writing plans/{id}.featureFlags under a rules constraint that permits only featureFlags+updatedAt). The two layers are deliberately NOT merged: FF_ answers "is it built and shipped?" → "coming soon"; entitlements answer "may this tier use it?"* → "upgrade to unlock". Merging them would make an unbuilt feature masquerade as a paywall. Scope exceeded, not just met</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="A6" s="49" t="inlineStr">
         <is>
           <t>R7</t>
         </is>
       </c>
-      <c r="B6" s="44" t="inlineStr">
+      <c r="B6" s="49" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="C6" s="44" t="inlineStr">
+      <c r="C6" s="49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D6" s="45" t="inlineStr">
+      <c r="D6" s="49" t="inlineStr">
         <is>
           <t>Project setup: Firebase, Polygon sub + keys, data-source verification</t>
         </is>
       </c>
-      <c r="E6" s="45" t="inlineStr">
+      <c r="E6" s="49" t="inlineStr">
         <is>
           <t>Polygon (Massive)</t>
         </is>
       </c>
-      <c r="F6" s="45" t="inlineStr">
+      <c r="F6" s="49" t="inlineStr">
         <is>
           <t>— (key/entitlement verification)</t>
         </is>
       </c>
-      <c r="G6" s="45" t="inlineStr">
-        <is>
-          <t>— *(setup)*</t>
-        </is>
-      </c>
-      <c r="H6" s="44" t="inlineStr">
+      <c r="G6" s="49" t="inlineStr">
+        <is>
+          <t>— (setup)</t>
+        </is>
+      </c>
+      <c r="H6" s="49" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="I6" s="45" t="inlineStr">
+      <c r="I6" s="49" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J6" s="45" t="inlineStr">
+      <c r="J6" s="49" t="inlineStr">
         <is>
           <t>Complete — all keys present and verified</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="46" t="inlineStr">
+      <c r="A7" s="50" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="B7" s="46" t="inlineStr">
+      <c r="B7" s="50" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="C7" s="46" t="inlineStr">
+      <c r="C7" s="50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D7" s="47" t="inlineStr">
+      <c r="D7" s="50" t="inlineStr">
         <is>
           <t>Run all sync jobs once; verify sync_meta + ops dashboard</t>
         </is>
       </c>
-      <c r="E7" s="47" t="inlineStr">
+      <c r="E7" s="50" t="inlineStr">
         <is>
           <t>multiple (all sync jobs)</t>
         </is>
       </c>
-      <c r="F7" s="47" t="inlineStr">
+      <c r="F7" s="50" t="inlineStr">
         <is>
           <t>— (21 jobs; see per-row endpoints)</t>
         </is>
       </c>
-      <c r="G7" s="47" t="inlineStr">
-        <is>
-          <t>— *(all sync jobs)*</t>
-        </is>
-      </c>
-      <c r="H7" s="46" t="inlineStr">
+      <c r="G7" s="50" t="inlineStr">
+        <is>
+          <t>— (all sync jobs)</t>
+        </is>
+      </c>
+      <c r="H7" s="50" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="I7" s="47" t="inlineStr">
+      <c r="I7" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J7" s="47" t="inlineStr">
-        <is>
-          <t>21/21 jobs run, sync_meta populated, monitor UI live</t>
+      <c r="J7" s="50" t="inlineStr">
+        <is>
+          <t>21/21 jobs run, sync_meta populated, monitor UI live. ⚠️ 2026-07-29 — deliverable's shape changed: the 21-job model was retired 2026-07-26 in favor of one sync-premarket cron (phased: profile warm → market-wide jobs → dynamic-universe compute → recap) plus on-demand fetch-on-miss for everything else. sync_meta still tracks whatever runs; "21/21" is no longer the right unit to verify against — re-check sync_meta against the new single-job phases, not the old per-job list.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="44" t="inlineStr">
+      <c r="A8" s="49" t="inlineStr">
         <is>
           <t>R9</t>
         </is>
       </c>
-      <c r="B8" s="44" t="inlineStr">
+      <c r="B8" s="49" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="C8" s="44" t="inlineStr">
+      <c r="C8" s="49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D8" s="45" t="inlineStr">
+      <c r="D8" s="49" t="inlineStr">
         <is>
           <t>Market Movers live (gainers/losers/unusual-vol/RVol/filter)</t>
         </is>
       </c>
-      <c r="E8" s="45" t="inlineStr">
+      <c r="E8" s="49" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F8" s="45" t="inlineStr">
+      <c r="F8" s="49" t="inlineStr">
         <is>
           <t>/v2/snapshot/…/{gainers,losers} + /v2/aggs/grouped/locale/us/market/stocks/{date}</t>
         </is>
       </c>
-      <c r="G8" s="45" t="inlineStr">
+      <c r="G8" s="49" t="inlineStr">
         <is>
           <t>Movers · gainers / losers / unusual-vol table</t>
         </is>
       </c>
-      <c r="H8" s="44" t="inlineStr">
+      <c r="H8" s="49" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I8" s="45" t="inlineStr">
+      <c r="I8" s="49" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J8" s="45" t="inlineStr">
+      <c r="J8" s="49" t="inlineStr">
         <is>
           <t>✅ 2026-07-21: MA-posture (real SMA50/200), week% (real 5-session change), tech-context (RSI/MACD/RS/RVOL) now live — added SMA/week fields to technical-indicators.job (rev 00019, ran for 238 tickers); catalyst now flags tickers with recent synced news ⬆ 100% on 2026-07-23: the catalyst field is now strictly honest — 'Recent news' (a real recent Polygon article exists for the ticker, via companies.newsCount) or 'No known catalyst'. The fabricated fallback to the hardcoded mock label ('Earnings beat', 'Guidance raise') was removed from the Movers screen, the Dashboard movers widget and the mover drawer — no row asserts an invented catalyst. Everything on this row is now Polygon-sourced with zero fabrication.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="46" t="inlineStr">
+      <c r="A9" s="50" t="inlineStr">
         <is>
           <t>R10</t>
         </is>
       </c>
-      <c r="B9" s="46" t="inlineStr">
+      <c r="B9" s="50" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="C9" s="46" t="inlineStr">
+      <c r="C9" s="50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D9" s="47" t="inlineStr">
+      <c r="D9" s="50" t="inlineStr">
         <is>
           <t>Market Heatmap live (sector %, tiles, summary)</t>
         </is>
       </c>
-      <c r="E9" s="47" t="inlineStr">
+      <c r="E9" s="50" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F9" s="47" t="inlineStr">
+      <c r="F9" s="50" t="inlineStr">
         <is>
           <t>/v2/aggs/grouped/locale/us/market/stocks/{date} (11 SPDR sector-ETF proxies)</t>
         </is>
       </c>
-      <c r="G9" s="47" t="inlineStr">
+      <c r="G9" s="50" t="inlineStr">
         <is>
           <t>Heatmap · sector treemap + tiles</t>
         </is>
       </c>
-      <c r="H9" s="46" t="inlineStr">
+      <c r="H9" s="50" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I9" s="47" t="inlineStr">
+      <c r="I9" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J9" s="47" t="inlineStr">
+      <c r="J9" s="50" t="inlineStr">
         <is>
           <t>✅ 2026-07-21: hover tooltip now reads live companies (price/RVOL/RS/MA-status); dead Stocks/S&amp;P-500 tab repurposed to a real Day%/Week% heat toggle (5-session change from technical-indicators.job, cap-weighted sector avg). S&amp;P-500 filter dropped — no constituent list available ⬆ 100% 2026-07-23: heatmap tiles now sample-labeled when no live sector data has synced; the dropped S&amp;P-500 filter was an out-of-scope extra (no constituent list on Starter), so the stated deliverable (sector %/tiles/summary) is fully met.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="44" t="inlineStr">
+      <c r="A10" s="49" t="inlineStr">
         <is>
           <t>R11</t>
         </is>
       </c>
-      <c r="B10" s="44" t="inlineStr">
+      <c r="B10" s="49" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="C10" s="44" t="inlineStr">
+      <c r="C10" s="49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D10" s="45" t="inlineStr">
+      <c r="D10" s="49" t="inlineStr">
         <is>
           <t>Dashboard core widgets live (AI card → R19)</t>
         </is>
       </c>
-      <c r="E10" s="45" t="inlineStr">
+      <c r="E10" s="49" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F10" s="45" t="inlineStr">
+      <c r="F10" s="49" t="inlineStr">
         <is>
           <t>/v2/aggs/grouped/locale/us/market/stocks/{date} (market-breadth)</t>
         </is>
       </c>
-      <c r="G10" s="45" t="inlineStr">
+      <c r="G10" s="49" t="inlineStr">
         <is>
           <t>Dashboard · core widgets (Market Pulse, internals, VIX)</t>
         </is>
       </c>
-      <c r="H10" s="44" t="inlineStr">
+      <c r="H10" s="49" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I10" s="45" t="inlineStr">
+      <c r="I10" s="49" t="inlineStr">
         <is>
           <t>AI card → R35 (Anthropic); Recaps → R28 — both separately tracked, not this row</t>
         </is>
       </c>
-      <c r="J10" s="45" t="inlineStr">
+      <c r="J10" s="49" t="inlineStr">
         <is>
           <t>✅ 2026-07-21: Market Internals + F&amp;G history now live from new market-breadth.job (176 days backfilled); VIX/Portfolio fake fallbacks removed (show — when absent) ⬆ 100% of the core-widget scope 2026-07-23. All dashboard widgets are live from Polygon; the 'What Matters Now' AI card is tracked in R35 (Anthropic — your planned purchase) and the Recaps card in R28, neither part of this row's widget deliverable.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="46" t="inlineStr">
+      <c r="A11" s="50" t="inlineStr">
         <is>
           <t>R13</t>
         </is>
       </c>
-      <c r="B11" s="46" t="inlineStr">
+      <c r="B11" s="50" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="C11" s="46" t="inlineStr">
+      <c r="C11" s="50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D11" s="47" t="inlineStr">
+      <c r="D11" s="50" t="inlineStr">
         <is>
           <t>Macro &amp; VIX live (econ calendar + dividends + VIX/yields)</t>
         </is>
       </c>
-      <c r="E11" s="47" t="inlineStr">
+      <c r="E11" s="50" t="inlineStr">
         <is>
           <t>Polygon + FRED (US-gov)</t>
         </is>
       </c>
-      <c r="F11" s="47" t="inlineStr">
+      <c r="F11" s="50" t="inlineStr">
         <is>
           <t>Polygon /fed/v1/treasury-yields + VIXY via /v2/aggs; FRED macro series (FredService). Not Finnhub.</t>
         </is>
       </c>
-      <c r="G11" s="47" t="inlineStr">
+      <c r="G11" s="50" t="inlineStr">
         <is>
           <t>Macro · VIX card, 10-yr yield, dividends</t>
         </is>
       </c>
-      <c r="H11" s="46" t="inlineStr">
+      <c r="H11" s="50" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I11" s="47" t="inlineStr">
+      <c r="I11" s="50" t="inlineStr">
         <is>
           <t>True spot VIX needs the Polygon Indices add-on (a purchase); VIXY proxy is the delivered, labeled solution</t>
         </is>
       </c>
-      <c r="J11" s="47" t="inlineStr">
-        <is>
-          <t>✅ 2026-07-21: Macro VIX card live via market_indices VIXY; dividend Month tab from live dividends. ⚠️ Correctness fix 2026-07-22 — the 10-year yield was previously WRONG, not merely proxied. market-indices.job.ts was publishing the TLT ETF price under the label "US10Y". TLT moves *inversely* to the yield it was labelled as, so the card showed the yield falling when it was rising. Now sourced from Polygon /fed/v1/treasury-yields — the real Treasury yield, isProxy:false, unit:"percent". Also new: dividend_history/{ticker} (241 docs) carrying full payment history, annual totals, TTM, derived yield, 5y CAGR and increase streak; and splits/{ticker} (241 docs) ⬆ 100% 2026-07-23: VIXY is the delivered, honestly-labeled (isProxy:true) proxy — consistent with the ETF proxies used for every index tile in this app. Spot VIX (I:VIX → 403) would need the Polygon Indices add-on, a future purchase like AI, not a gap in the delivered solution.</t>
+      <c r="J11" s="50" t="inlineStr">
+        <is>
+          <t>✅ 2026-07-21: Macro VIX card live via market_indices VIXY; dividend Month tab from live dividends. ⚠️ Correctness fix 2026-07-22 — the 10-year yield was previously WRONG, not merely proxied. market-indices.job.ts was publishing the TLT ETF price under the label "US10Y". TLT moves inversely to the yield it was labelled as, so the card showed the yield falling when it was rising. Now sourced from Polygon /fed/v1/treasury-yields — the real Treasury yield, isProxy:false, unit:"percent". Also new: dividend_history/{ticker} (241 docs) carrying full payment history, annual totals, TTM, derived yield, 5y CAGR and increase streak; and splits/{ticker} (241 docs — ⚠️ pre-reset snapshot, see 2026-07-29 note above; the 2026-07-26 DB reset deleted market-data collections, so this count no longer reflects current Firestore state, only that the mechanism produced this many docs before the reset) ⬆ 100% 2026-07-23: VIXY is the delivered, honestly-labeled (isProxy:true) proxy — consistent with the ETF proxies used for every index tile in this app. Spot VIX (I:VIX → 403) would need the Polygon Indices add-on, a future purchase like AI, not a gap in the delivered solution.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="44" t="inlineStr">
+      <c r="A12" s="49" t="inlineStr">
         <is>
           <t>R14</t>
         </is>
       </c>
-      <c r="B12" s="44" t="inlineStr">
+      <c r="B12" s="49" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="C12" s="44" t="inlineStr">
+      <c r="C12" s="49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D12" s="45" t="inlineStr">
+      <c r="D12" s="49" t="inlineStr">
         <is>
           <t>IPOs live (calendar + offer price)</t>
         </is>
       </c>
-      <c r="E12" s="45" t="inlineStr">
+      <c r="E12" s="49" t="inlineStr">
         <is>
           <t>Polygon (only)</t>
         </is>
       </c>
-      <c r="F12" s="45" t="inlineStr">
+      <c r="F12" s="49" t="inlineStr">
         <is>
           <t>/vX/reference/ipos. Finnhub fallback removed — not redistribution-licensed; prod already ran fallback=none.</t>
         </is>
       </c>
-      <c r="G12" s="45" t="inlineStr">
+      <c r="G12" s="49" t="inlineStr">
         <is>
           <t>IPOs · IPO calendar + aftermarket perf</t>
         </is>
       </c>
-      <c r="H12" s="44" t="inlineStr">
+      <c r="H12" s="49" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I12" s="45" t="inlineStr">
+      <c r="I12" s="49" t="inlineStr">
         <is>
           <t>SPAC units / brand-new tickers with no Polygon bars show "—" (honest, not mock)</t>
         </is>
       </c>
-      <c r="J12" s="45" t="inlineStr">
+      <c r="J12" s="49" t="inlineStr">
         <is>
           <t>⬆ Corrected 2026-07-23 — the 'falls back to mock' note was stale. ipos.job.ts already derives day-1 and since-IPO returns from Polygon /v2/aggs (getAggsRange) — verified live: 40/52 IPO docs carry real aftermarket performance. The mock RECENT_IPOS renders only when the live collection is empty (it isn't). Polygon-only, no non-redistributable data. ⬆ 100% 2026-07-23.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="46" t="inlineStr">
+      <c r="A13" s="50" t="inlineStr">
         <is>
           <t>R15</t>
         </is>
       </c>
-      <c r="B13" s="46" t="inlineStr">
+      <c r="B13" s="50" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="C13" s="46" t="inlineStr">
+      <c r="C13" s="50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D13" s="47" t="inlineStr">
+      <c r="D13" s="50" t="inlineStr">
         <is>
           <t>Commentary/News live (aggregated feed + tags + drawer)</t>
         </is>
       </c>
-      <c r="E13" s="47" t="inlineStr">
+      <c r="E13" s="50" t="inlineStr">
         <is>
           <t>Polygon (only)</t>
         </is>
       </c>
-      <c r="F13" s="47" t="inlineStr">
+      <c r="F13" s="50" t="inlineStr">
         <is>
           <t>/v2/reference/news. Finnhub dropped from the news feed — not redistribution-licensed (was NEWS_SOURCE=aggregate).</t>
         </is>
       </c>
-      <c r="G13" s="47" t="inlineStr">
+      <c r="G13" s="50" t="inlineStr">
         <is>
           <t>Commentary · aggregated news feed</t>
         </is>
       </c>
-      <c r="H13" s="46" t="inlineStr">
+      <c r="H13" s="50" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I13" s="47" t="inlineStr">
+      <c r="I13" s="50" t="inlineStr">
         <is>
           <t>Narrative "before the bell / after the close" briefs are AI content → R35 (Anthropic), honestly SampleBadge-labeled</t>
         </is>
       </c>
-      <c r="J13" s="47" t="inlineStr">
+      <c r="J13" s="50" t="inlineStr">
         <is>
           <t>Those sub-feeds have no live source; main feed is live ⬆ 100% of the DATA scope 2026-07-23: the news feed (Polygon /v2/reference/news) and extended-hours moves (Polygon /v3/snapshot via useExtendedHours) are live; the two narrative brief cards are AI-generated content, labeled and tracked under R35 (Anthropic). No non-AI gap remains.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="44" t="inlineStr">
+      <c r="A14" s="49" t="inlineStr">
         <is>
           <t>R16</t>
         </is>
       </c>
-      <c r="B14" s="44" t="inlineStr">
+      <c r="B14" s="49" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="C14" s="44" t="inlineStr">
+      <c r="C14" s="49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D14" s="45" t="inlineStr">
+      <c r="D14" s="49" t="inlineStr">
         <is>
           <t>Sector Themes live (per-stock prices + theme perf)</t>
         </is>
       </c>
-      <c r="E14" s="45" t="inlineStr">
+      <c r="E14" s="49" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F14" s="45" t="inlineStr">
+      <c r="F14" s="49" t="inlineStr">
         <is>
           <t>/v3/reference/tickers (companies prices)</t>
         </is>
       </c>
-      <c r="G14" s="45" t="inlineStr">
+      <c r="G14" s="49" t="inlineStr">
         <is>
           <t>Themes · sector-theme baskets</t>
         </is>
       </c>
-      <c r="H14" s="44" t="inlineStr">
+      <c r="H14" s="49" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I14" s="45" t="inlineStr">
+      <c r="I14" s="49" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J14" s="45" t="inlineStr">
-        <is>
-          <t>Theme baskets are static config (fine); prices live when matched ⬆ 100% 2026-07-23: matched tickers show live Polygon prices; unmatched (outside the synced universe) are SampleBadge-labeled with a live/total count. Theme baskets are static config by design.</t>
+      <c r="J14" s="49" t="inlineStr">
+        <is>
+          <t>Theme baskets are static config (fine); prices live when matched ⬆ 100% 2026-07-23: matched tickers show live Polygon prices; unmatched (outside the synced universe) are SampleBadge-labeled with a live/total count. Theme baskets are static config by design. ❓ Open question, 2026-07-29 — not a stale citation, a genuine unknown: "synced universe" pre-2026-07-26 meant the fixed 241-ticker list; that list is now retired in favor of a dynamic universe (only tickers actually touched by tape/watchlist/portfolio/ticker_usage). If a theme basket's tickers aren't in that dynamic set, they'd show as SampleBadge/unmatched until a user searches them (triggering on-demand fetch) rather than being pre-warmed. Whether that changes the live/total ratio in practice needs a real check against production — not asserted here either way; row % left at 100% pending that check.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="46" t="inlineStr">
+      <c r="A15" s="50" t="inlineStr">
         <is>
           <t>R17</t>
         </is>
       </c>
-      <c r="B15" s="46" t="inlineStr">
+      <c r="B15" s="50" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="C15" s="46" t="inlineStr">
+      <c r="C15" s="50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D15" s="47" t="inlineStr">
+      <c r="D15" s="50" t="inlineStr">
         <is>
           <t>Company-name search (nameLower/tokens)</t>
         </is>
       </c>
-      <c r="E15" s="47" t="inlineStr">
+      <c r="E15" s="50" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F15" s="47" t="inlineStr">
+      <c r="F15" s="50" t="inlineStr">
         <is>
           <t>/v3/reference/tickers</t>
         </is>
       </c>
-      <c r="G15" s="47" t="inlineStr">
+      <c r="G15" s="50" t="inlineStr">
         <is>
           <t>Search (⌘K / shell) · company-name search</t>
         </is>
       </c>
-      <c r="H15" s="46" t="inlineStr">
+      <c r="H15" s="50" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I15" s="47" t="inlineStr">
+      <c r="I15" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J15" s="47" t="inlineStr">
-        <is>
-          <t>ticker-universe writes nameLower/searchTokens; ⌘K search live ⬆ 100% 2026-07-23: company-name search is live over the full ticker universe (nameLower/searchTokens). ⬆ 2026-07-23: ⌘K search results now overlay live delayed prices (Polygon /live/snapshot via useSnapshotQuotes, polled only while the palette is open) on top of the EOD companies price.</t>
+      <c r="J15" s="50" t="inlineStr">
+        <is>
+          <t>ticker-universe writes nameLower/searchTokens; ⌘K search live ⬆ 100% 2026-07-23: company-name search is live over the full ticker universe (nameLower/searchTokens). ⬆ 2026-07-23: ⌘K search results now overlay live delayed prices (Polygon /live/snapshot via useSnapshotQuotes, polled only while the palette is open) on top of the EOD companies price. ⚠️ 2026-07-29 — mechanism superseded: the nameLower/searchTokens-on-tickers approach above was retired 2026-07-26; the tickers collection is now retired entirely and search runs over the in-memory GET /live/search index (full ~13k Polygon universe, per-instance, refreshed daily, substring matching, zero Firestore reads). Row stays 100% — search is still live, arguably improved (substring match vs. prefix-only) — but re-point any future audit at /live/search, not tickers.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="44" t="inlineStr">
+      <c r="A16" s="49" t="inlineStr">
         <is>
           <t>R19</t>
         </is>
       </c>
-      <c r="B16" s="44" t="inlineStr">
+      <c r="B16" s="49" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="C16" s="44" t="inlineStr">
+      <c r="C16" s="49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D16" s="45" t="inlineStr">
+      <c r="D16" s="49" t="inlineStr">
         <is>
           <t>Portfolio Pulse live (holdings + prices + P&amp;L + totals)</t>
         </is>
       </c>
-      <c r="E16" s="45" t="inlineStr">
+      <c r="E16" s="49" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F16" s="45" t="inlineStr">
+      <c r="F16" s="49" t="inlineStr">
         <is>
           <t>/v3/snapshot · /v2/snapshot (holding prices)</t>
         </is>
       </c>
-      <c r="G16" s="45" t="inlineStr">
+      <c r="G16" s="49" t="inlineStr">
         <is>
           <t>Portfolio · holdings + prices + P&amp;L</t>
         </is>
       </c>
-      <c r="H16" s="44" t="inlineStr">
+      <c r="H16" s="49" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I16" s="45" t="inlineStr">
+      <c r="I16" s="49" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J16" s="45" t="inlineStr">
+      <c r="J16" s="49" t="inlineStr">
         <is>
           <t>Real holdings + live prices + P&amp;L all work; fallback is cosmetic ⬆ 100% 2026-07-23: the Portfolio Pulse SCREEN uses real holdings + live Polygon prices + P&amp;L, sample-labeled when a holding is outside the synced universe. The $128,430 figure is on the pre-login MARKETING landing (page.tsx), a showcase — not the app. ⬆ 2026-07-23 — two upgrades. (1) Holding prices and the portfolio total (Σ shares×price) + day P&amp;L now track live delayed prices (Polygon /live/snapshot), not the once-a-day EOD write. (2) CRUD gap fixed: share quantity was hardcoded to 10 with no editor — added a Shares input to the add form and an editable position strip for the selected holding, both persisted to Firestore, so the total reflects real share counts. The $128,430 figure remains only on the marketing landing.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="46" t="inlineStr">
+      <c r="A17" s="50" t="inlineStr">
         <is>
           <t>R20</t>
         </is>
       </c>
-      <c r="B17" s="46" t="inlineStr">
+      <c r="B17" s="50" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="C17" s="46" t="inlineStr">
+      <c r="C17" s="50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D17" s="47" t="inlineStr">
+      <c r="D17" s="50" t="inlineStr">
         <is>
           <t>Watchlist live (persistence + prices + AI summary)</t>
         </is>
       </c>
-      <c r="E17" s="47" t="inlineStr">
+      <c r="E17" s="50" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F17" s="47" t="inlineStr">
+      <c r="F17" s="50" t="inlineStr">
         <is>
           <t>/v3/snapshot (watchlist prices)</t>
         </is>
       </c>
-      <c r="G17" s="47" t="inlineStr">
+      <c r="G17" s="50" t="inlineStr">
         <is>
           <t>Watchlist · prices + persistence</t>
         </is>
       </c>
-      <c r="H17" s="46" t="inlineStr">
+      <c r="H17" s="50" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I17" s="47" t="inlineStr">
+      <c r="I17" s="50" t="inlineStr">
         <is>
           <t>The "AI summary" is AI content → R39 (Anthropic); persistence + prices are done and labeled</t>
         </is>
       </c>
-      <c r="J17" s="47" t="inlineStr">
+      <c r="J17" s="50" t="inlineStr">
         <is>
           <t>AI intentionally deferred to R34/R39; persistence + prices done ⬆ 100% of the non-AI scope 2026-07-23: watchlist persistence + live Polygon prices are done and sample-labeled; the 'AI summary' is tracked under R39 (Anthropic — your planned purchase). ⬆ 2026-07-23: watchlist prices now overlay live delayed prices (Polygon /live/snapshot) on the EOD price. CRUD verified: add/remove persist via Firestore arrayUnion/arrayRemove on users/{uid}/watchlists/default. (AI summary still R39 — Anthropic.)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="44" t="inlineStr">
+      <c r="A18" s="49" t="inlineStr">
         <is>
           <t>R21</t>
         </is>
       </c>
-      <c r="B18" s="44" t="inlineStr">
+      <c r="B18" s="49" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="C18" s="44" t="inlineStr">
+      <c r="C18" s="49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D18" s="45" t="inlineStr">
+      <c r="D18" s="49" t="inlineStr">
         <is>
           <t>Empty-states + graceful fallback polish (cross-screen)</t>
         </is>
       </c>
-      <c r="E18" s="45" t="inlineStr">
+      <c r="E18" s="49" t="inlineStr">
         <is>
           <t>— (cross-screen)</t>
         </is>
       </c>
-      <c r="F18" s="45" t="inlineStr">
+      <c r="F18" s="49" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="45" t="inlineStr">
-        <is>
-          <t>— *(cross-screen empty states)*</t>
-        </is>
-      </c>
-      <c r="H18" s="44" t="inlineStr">
+      <c r="G18" s="49" t="inlineStr">
+        <is>
+          <t>— (cross-screen empty states)</t>
+        </is>
+      </c>
+      <c r="H18" s="49" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I18" s="45" t="inlineStr">
+      <c r="I18" s="49" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J18" s="45" t="inlineStr">
+      <c r="J18" s="49" t="inlineStr">
         <is>
           <t>Only IPOs/Options/Insider label mock data; pattern not applied app-wide ⬆ 100% 2026-07-23: the sample-labeling pattern is now applied across every W1–W3 data screen — movers, screener, portfolio, watchlist and heatmap gained a &lt;SampleBadge&gt; (shown when data isn't fully live), joining the already-labeled commentary, earnings, insider, macro, recap, themes and ipos. No W1–W3 screen silently shows mock. (analyst/options/stock are labeled within their own rows R41/R32/R24.)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="46" t="inlineStr">
+      <c r="A19" s="50" t="inlineStr">
         <is>
           <t>R23</t>
         </is>
       </c>
-      <c r="B19" s="46" t="inlineStr">
+      <c r="B19" s="50" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="C19" s="46" t="inlineStr">
+      <c r="C19" s="50" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D19" s="47" t="inlineStr">
+      <c r="D19" s="50" t="inlineStr">
         <is>
           <t>ENABLER: backfill ohlcv_bars + compute jobs</t>
         </is>
       </c>
-      <c r="E19" s="47" t="inlineStr">
+      <c r="E19" s="50" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F19" s="47" t="inlineStr">
+      <c r="F19" s="50" t="inlineStr">
         <is>
           <t>/v2/aggs/ticker/{sym}/range/1/day/… + /range/{5,30}/minute/…</t>
         </is>
       </c>
-      <c r="G19" s="47" t="inlineStr">
-        <is>
-          <t>— *(enabler; feeds Stock-detail charts)*</t>
-        </is>
-      </c>
-      <c r="H19" s="46" t="inlineStr">
+      <c r="G19" s="50" t="inlineStr">
+        <is>
+          <t>— (enabler; feeds Stock-detail charts)</t>
+        </is>
+      </c>
+      <c r="H19" s="50" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="I19" s="47" t="inlineStr">
+      <c r="I19" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J19" s="47" t="inlineStr">
-        <is>
-          <t>Ahead of schedule — all 5 compute jobs green. Deepened 2026-07-22: ohlcv_bars now holds ~299,552 documents spanning the full 5-year window (was ~300 days). Raising the backfill constant alone did nothing — lastSyncedThrough only ever advances — so stock-history.job.ts gained an earliestSyncedFrom watermark that fills history backwards as well as forwards, clamped to the plan's rolling 5-year edge. vwap now persisted per bar. Also new: intraday_bars (474 docs, 5-min + 30-min, one doc per ticker/resolution holding an array of bars)</t>
+      <c r="J19" s="50" t="inlineStr">
+        <is>
+          <t>Ahead of schedule — all 5 compute jobs green. Deepened 2026-07-22: ohlcv_bars now holds ~299,552 documents spanning the full 5-year window (was ~300 days). Raising the backfill constant alone did nothing — lastSyncedThrough only ever advances — so stock-history.job.ts gained an earliestSyncedFrom watermark that fills history backwards as well as forwards, clamped to the plan's rolling 5-year edge. vwap now persisted per bar. Also new: intraday_bars (474 docs, 5-min + 30-min, one doc per ticker/resolution holding an array of bars) — ⚠️ 2026-07-29 — deliverable re-scoped, not just re-counted: this row's original scope (backfill a fixed 241-ticker universe to 5 years) was superseded 2026-07-26. Bars are now on-demand and incremental, keyed in stock_bars/ (_1min/_5min/_30min/_daily, widen-in-place); a full 5-year series is never pre-downloaded for a ticker nobody has requested. ohlcv_bars/intraday_bars remain only as the internal substrate the indicator jobs read, not the client path, and the fixed 241-ticker list is retired in favor of the dynamic (actually-used) universe. The new deliverable — bars available on request for any ticker at any timeframe, with zero re-download of already-synced ranges — is still met, so this stays 100%, but "backfill the fixed universe" as originally written no longer describes what the system does.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="44" t="inlineStr">
+      <c r="A20" s="49" t="inlineStr">
         <is>
           <t>R24</t>
         </is>
       </c>
-      <c r="B20" s="44" t="inlineStr">
+      <c r="B20" s="49" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="C20" s="44" t="inlineStr">
+      <c r="C20" s="49" t="inlineStr">
         <is>
           <t>🔵→</t>
         </is>
       </c>
-      <c r="D20" s="45" t="inlineStr">
+      <c r="D20" s="49" t="inlineStr">
         <is>
           <t>Stock Detail live (charts/RSI-MACD/fundamentals/52-wk/consensus/news/insider)</t>
         </is>
       </c>
-      <c r="E20" s="45" t="inlineStr">
+      <c r="E20" s="49" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F20" s="45" t="inlineStr">
+      <c r="F20" s="49" t="inlineStr">
         <is>
           <t>/v2/aggs/ticker/{sym}/range/…, /vX/reference/financials, /v1/related-companies/{sym}</t>
         </is>
       </c>
-      <c r="G20" s="45" t="inlineStr">
+      <c r="G20" s="49" t="inlineStr">
         <is>
           <t>Stock detail · chart / RSI-MACD / financials / 52-wk / peers</t>
         </is>
       </c>
-      <c r="H20" s="44" t="inlineStr">
+      <c r="H20" s="49" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I20" s="45" t="inlineStr">
+      <c r="I20" s="49" t="inlineStr">
         <is>
           <t>Analyst consensus uses FMP (required — Polygon has no analyst product on Starter); true per-firm analyst actions → R41 (Benzinga add-on). AI thesis/risk block → R38 (Anthropic). Both separately tracked</t>
         </is>
       </c>
-      <c r="J20" s="45" t="inlineStr">
-        <is>
-          <t>⬆ Raised from 80% on 2026-07-22 — the previous entry mis-diagnosed the gap. The old note said 1D/1W needed intraday bars and 5Y needed 5-year history, implying a data-plan block. That was wrong: both were authorized on the existing Polygon Stocks Starter plan all along (intraday aggregates ✅, 5-year rolling history ✅ — re-probed live). It was a sync gap, not a plan gap — we simply had not pulled them. Now synced: intraday-bars.job.ts (new) feeds 1D/1W, and the 5-year backfill (R23) feeds 5Y. All 7 chart timeframes now read real bars via useChartBars. Also real: full financial statements, 52-wk high/low + %-from, SMA/EMA ladders (10/20/30/50/100/200), 90-point rsi14Series, VWAP, peers (/v1/related-companies), dividend yield + DPS. No synthetic timeframes remain ⬆ 100% 2026-07-23 — all remaining fabrications on the screen removed. Revenue (TTM) now = last 4 real quarters (Polygon financials); the dead finRows panel and its fabricated FCF/debt are gone; the 'recent EPS' rows and the EPS-surprise pane now read real fin.epsHistory (beat/miss only where a real estimate exists, else 'no est.'); the technical ratings are computed from real indicators — Moving Averages from price vs each real SMA/EMA, Oscillators from real RSI(14)+MACD; and a header &lt;SampleBadge&gt; flags any ticker outside the synced universe (covering the RSI/SMA/vol/pivot/52wk fallbacks). The analyst consensus panel is FMP-backed — kept per decision; it is a consensus snapshot, and per-firm upgrades/downgrades remain R41 (Benzinga). The AI thesis is R38 (Anthropic). Charts, RSI/MACD, full financial statements, 52-week, news and insider (SEC) were already live. ⬆ 2026-07-24 deepened (still 100%): the header price + chart now use the shared live-price subscription (delayed snapshot) instead of the once-a-day close, and the fundamentals gained Quarterly / Yearly tabs (annual financials). The TradingView compare surface was removed from the shipped page — the stock chart is now our own Polygon-backed CandleChart, last bar tracking the live price.</t>
+      <c r="J20" s="49" t="inlineStr">
+        <is>
+          <t>⬆ Raised from 80% on 2026-07-22 — the previous entry mis-diagnosed the gap. The old note said 1D/1W needed intraday bars and 5Y needed 5-year history, implying a data-plan block. That was wrong: both were authorized on the existing Polygon Stocks Starter plan all along (intraday aggregates ✅, 5-year rolling history ✅ — re-probed live). It was a sync gap, not a plan gap — we simply had not pulled them. Now synced: intraday-bars.job.ts (new) feeds 1D/1W, and the 5-year backfill (R23) feeds 5Y. All 7 chart timeframes now read real bars via useChartBars. Also real: full financial statements, 52-wk high/low + %-from, SMA/EMA ladders (10/20/30/50/100/200), 90-point rsi14Series, VWAP, peers (/v1/related-companies), dividend yield + DPS. No synthetic timeframes remain ⬆ 100% 2026-07-23 — all remaining fabrications on the screen removed. Revenue (TTM) now = last 4 real quarters (Polygon financials); the dead finRows panel and its fabricated FCF/debt are gone; the 'recent EPS' rows and the EPS-surprise pane now read real fin.epsHistory (beat/miss only where a real estimate exists, else 'no est.'); the technical ratings are computed from real indicators — Moving Averages from price vs each real SMA/EMA, Oscillators from real RSI(14)+MACD; and a header &lt;SampleBadge&gt; flags any ticker outside the synced universe (covering the RSI/SMA/vol/pivot/52wk fallbacks). The analyst consensus panel is FMP-backed — kept per decision; it is a consensus snapshot, and per-firm upgrades/downgrades remain R41 (Benzinga). The AI thesis is R38 (Anthropic). Charts, RSI/MACD, full financial statements, 52-week, news and insider (SEC) were already live. ⬆ 2026-07-24 deepened (still 100%): the header price + chart now use the shared live-price subscription (delayed snapshot) instead of the once-a-day close, and the fundamentals gained Quarterly / Yearly tabs (annual financials). The TradingView compare surface was removed from the shipped page — the stock chart is now our own Polygon-backed CandleChart, last bar tracking the live price. ⚠️ 2026-07-29: as of 2026-07-26 the chart's data source is GET /live/bars?ticker&amp;tf (on-demand, Firestore-cached with TTL, stock_bars/ storage) rather than direct ohlcv_bars/intraday_bars reads — see R23's note. Functionally equivalent (all 7 timeframes still real), just a different read path; not independently re-verified against live production this pass.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="46" t="inlineStr">
+      <c r="A21" s="50" t="inlineStr">
         <is>
           <t>R25</t>
         </is>
       </c>
-      <c r="B21" s="46" t="inlineStr">
+      <c r="B21" s="50" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="C21" s="46" t="inlineStr">
+      <c r="C21" s="50" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D21" s="47" t="inlineStr">
+      <c r="D21" s="50" t="inlineStr">
         <is>
           <t>Screener live (filters + Tech Rating + RVOL + growth/margin)</t>
         </is>
       </c>
-      <c r="E21" s="47" t="inlineStr">
+      <c r="E21" s="50" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F21" s="47" t="inlineStr">
+      <c r="F21" s="50" t="inlineStr">
         <is>
           <t>/v3/reference/tickers + /vX/reference/financials</t>
         </is>
       </c>
-      <c r="G21" s="47" t="inlineStr">
+      <c r="G21" s="50" t="inlineStr">
         <is>
           <t>Screener · filters + Tech Rating + RVOL</t>
         </is>
       </c>
-      <c r="H21" s="46" t="inlineStr">
+      <c r="H21" s="50" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I21" s="47" t="inlineStr">
+      <c r="I21" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J21" s="47" t="inlineStr">
-        <is>
-          <t>Core overlay from companies live; a few filters never implemented ⬆ 100% 2026-07-23: the three dead no-op filter checkboxes — Above 50 &amp; 200-DMA, RSI 40–70, Price &gt; $5 — are now wired to real companies technicals (price/sma50/sma200/rsi14 from technical-indicators.job), with save/restore + reset. No no-op filter remains; every control filters on real Polygon-derived data. Verified against prod: of 241 priced companies, 114 pass the DMA filter, 211 RSI 40–70, 239 price&gt;$5.</t>
+      <c r="J21" s="50" t="inlineStr">
+        <is>
+          <t>Core overlay from companies live; a few filters never implemented ⬆ 100% 2026-07-23: the three dead no-op filter checkboxes — Above 50 &amp; 200-DMA, RSI 40–70, Price &gt; $5 — are now wired to real companies technicals (price/sma50/sma200/rsi14 from technical-indicators.job), with save/restore + reset. No no-op filter remains; every control filters on real Polygon-derived data. Verified against prod: of 241 priced companies, 114 pass the DMA filter, 211 RSI 40–70, 239 price&gt;$5. ❓ Open question, 2026-07-29 — not a stale citation, a genuine unknown: those 241 companies were the fixed pre-synced universe; per-ticker compute jobs (technical-indicators etc.) now run "over the dynamic universe" (only actually-used tickers, see the ON-DEMAND DATA LAYER block), and Firestore was reset empty on 2026-07-26. Screener's core value is scanning broadly — whether it still has a wide-enough pool of computed companies docs to screen against (vs. only whatever's been touched so far) is unverified from here and should be checked against production before trusting this row's 100%.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="44" t="inlineStr">
+      <c r="A22" s="49" t="inlineStr">
         <is>
           <t>R26</t>
         </is>
       </c>
-      <c r="B22" s="44" t="inlineStr">
+      <c r="B22" s="49" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="C22" s="44" t="inlineStr">
+      <c r="C22" s="49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D22" s="45" t="inlineStr">
+      <c r="D22" s="49" t="inlineStr">
         <is>
           <t>Dashboard Fear &amp; Greed gauge live</t>
         </is>
       </c>
-      <c r="E22" s="45" t="inlineStr">
+      <c r="E22" s="49" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F22" s="45" t="inlineStr">
+      <c r="F22" s="49" t="inlineStr">
         <is>
           <t>/v2/aggs/range (SPY/TLT/VIXY) + /v2/aggs/grouped (breadth)</t>
         </is>
       </c>
-      <c r="G22" s="45" t="inlineStr">
+      <c r="G22" s="49" t="inlineStr">
         <is>
           <t>Dashboard · Fear &amp; Greed gauge</t>
         </is>
       </c>
-      <c r="H22" s="44" t="inlineStr">
+      <c r="H22" s="49" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I22" s="45" t="inlineStr">
+      <c r="I22" s="49" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J22" s="45" t="inlineStr">
+      <c r="J22" s="49" t="inlineStr">
         <is>
           <t>⬆ 100% on 2026-07-23 — the composite methodology is now real. The fear-greed.job computes the true 4-component composite (momentum from SPY vs its 125-day MA, safe-haven from SPY−TLT 20-day return spread, volatility from VIXY vs its 50-day MA, breadth from grouped-daily advancers) for both the live value and a backfilled market_sentiment_history/{date} series (25 trading days, verified). The dashboard sparkline now reads that real composite history instead of the breadth-only proxy. The earlier missing-rule bug (gauge silently rendering a hardcoded 62) was fixed on 07-22; market_sentiment_history rule added and released 07-23.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="46" t="inlineStr">
+      <c r="A23" s="50" t="inlineStr">
         <is>
           <t>R28</t>
         </is>
       </c>
-      <c r="B23" s="46" t="inlineStr">
+      <c r="B23" s="50" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="C23" s="46" t="inlineStr">
+      <c r="C23" s="50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D23" s="47" t="inlineStr">
+      <c r="D23" s="50" t="inlineStr">
         <is>
           <t>Recaps EOD data job</t>
         </is>
       </c>
-      <c r="E23" s="47" t="inlineStr">
+      <c r="E23" s="50" t="inlineStr">
         <is>
           <t>Polygon (composed)</t>
         </is>
       </c>
-      <c r="F23" s="47" t="inlineStr">
+      <c r="F23" s="50" t="inlineStr">
         <is>
           <t>Composes market_indices / market_movers / sectors / market_breadth → recaps/{date}</t>
         </is>
       </c>
-      <c r="G23" s="47" t="inlineStr">
+      <c r="G23" s="50" t="inlineStr">
         <is>
           <t>Recap · end-of-day recap</t>
         </is>
       </c>
-      <c r="H23" s="46" t="inlineStr">
+      <c r="H23" s="50" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I23" s="47" t="inlineStr">
+      <c r="I23" s="50" t="inlineStr">
         <is>
           <t>AI prose lead + news briefing → R36 (Anthropic), separately tracked</t>
         </is>
       </c>
-      <c r="J23" s="47" t="inlineStr">
-        <is>
-          <t>⬆ 0% → 100% on 2026-07-23. New recaps.job (cron 45 18 * * 1-5, Scheduler sync-recaps registered) freezes each session's indices, top gainers/losers, sector leaders/laggards and market internals (advancers/decliners/breadth/TRIN/up-down volume) into one dated snapshot — Polygon-derived, no extra vendor call. recap.tsx now renders the live recaps/{date} doc: hero index tiles, Biggest Movers, Market Internals and the drawer A/D bar are real; the fabricated 'extended breadth' block (NYSE TICK / McClellan / Put-Call — not available from Polygon) was deleted. Verified: recaps/2026-07-21 written with 9 indices, 6+6 movers, 3+3 sectors, real internals. The prose lead + news briefing remain AI narrative → R36 (Anthropic, your planned purchase), the only recap sub-part not part of this data-job row.</t>
+      <c r="J23" s="50" t="inlineStr">
+        <is>
+          <t>⬆ 0% → 100% on 2026-07-23. New recaps.job (cron 45 18   1-5, Scheduler sync-recaps registered) freezes each session's indices, top gainers/losers, sector leaders/laggards and market internals (advancers/decliners/breadth/TRIN/up-down volume) into one dated snapshot — Polygon-derived, no extra vendor call. recap.tsx now renders the live recaps/{date} doc: hero index tiles, Biggest Movers, Market Internals and the drawer A/D bar are real; the fabricated 'extended breadth' block (NYSE TICK / McClellan / Put-Call — not available from Polygon) was deleted. Verified: recaps/2026-07-21 written with 9 indices, 6+6 movers, 3+3 sectors, real internals. The prose lead + news briefing remain AI narrative → R36 (Anthropic, your planned purchase), the only recap sub-part not part of this data-job row.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="44" t="inlineStr">
+      <c r="A24" s="49" t="inlineStr">
         <is>
           <t>R29</t>
         </is>
       </c>
-      <c r="B24" s="44" t="inlineStr">
+      <c r="B24" s="49" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="C24" s="44" t="inlineStr">
+      <c r="C24" s="49" t="inlineStr">
         <is>
           <t>🔵→</t>
         </is>
       </c>
-      <c r="D24" s="45" t="inlineStr">
+      <c r="D24" s="49" t="inlineStr">
         <is>
           <t>10-quarter EPS history (quarterly financials + wire)</t>
         </is>
       </c>
-      <c r="E24" s="45" t="inlineStr">
+      <c r="E24" s="49" t="inlineStr">
         <is>
           <t>Polygon (actuals) — estimates need Benzinga add-on</t>
         </is>
       </c>
-      <c r="F24" s="45" t="inlineStr">
+      <c r="F24" s="49" t="inlineStr">
         <is>
           <t>Polygon /vX/reference/financials (actuals). Estimate feed: Polygon Benzinga Earnings add-on (not on current plan)</t>
         </is>
       </c>
-      <c r="G24" s="45" t="inlineStr">
+      <c r="G24" s="49" t="inlineStr">
         <is>
           <t>Earnings hub · EPS &amp; Sales / Income statement</t>
         </is>
       </c>
-      <c r="H24" s="44" t="inlineStr">
+      <c r="H24" s="49" t="inlineStr">
         <is>
           <t>90% ⬇</t>
         </is>
       </c>
-      <c r="I24" s="45" t="inlineStr">
+      <c r="I24" s="49" t="inlineStr">
         <is>
           <t>EPS estimates — the forward/estimate side has no redistributable source on the current plan. FMP/Finnhub estimates exist in code but are NOT licensed for redistribution, so they must not ship to users</t>
         </is>
       </c>
-      <c r="J24" s="45" t="inlineStr">
-        <is>
-          <t>⬇ Recapped from 98% → 90% on 2026-07-23 to reflect the redistribution constraint honestly. The actuals are 100% Polygon and redistributable: 10 real quarters of EPS from /vX/reference/financials (~228 tickers), plus full balance sheet, cash flow, margins and current ratio — a complete fundamentals panel. The estimate overlay (actual-vs-estimate beat/miss) is the only gap: the only sources wired are FMP/Finnhub, which are not redistributable, so per the Polygon-only policy they cannot be served. A redistribution-legal estimate feed = Polygon's Benzinga Earnings &amp; Estimates add-on (a paid add-on to the current plan, tracked with R41/R42). Until purchased, estimates stay unshipped and this row is capped below 100%. ⬆ 2026-07-24 — actuals scope widened again (row still 90%, gap unchanged): financials now also carry 8 annual fiscal years (income/balance/cash-flow via timeframe=annual), so the earnings hub gained Quarterly / Yearly tabs on both EPS &amp; Sales history and the Income statement (actuals only, chart removed). The 90% cap is unmoved because it reflects the missing *estimate* feed, not the actuals.</t>
+      <c r="J24" s="49" t="inlineStr">
+        <is>
+          <t>⬇ Recapped from 98% → 90% on 2026-07-23 to reflect the redistribution constraint honestly. The actuals are 100% Polygon and redistributable: 10 real quarters of EPS from /vX/reference/financials (~228 tickers), plus full balance sheet, cash flow, margins and current ratio — a complete fundamentals panel. The estimate overlay (actual-vs-estimate beat/miss) is the only gap: the only sources wired are FMP/Finnhub, which are not redistributable, so per the Polygon-only policy they cannot be served. A redistribution-legal estimate feed = Polygon's Benzinga Earnings &amp; Estimates add-on (a paid add-on to the current plan, tracked with R41/R42). Until purchased, estimates stay unshipped and this row is capped below 100%. ⬆ 2026-07-24 — actuals scope widened again (row still 90%, gap unchanged): financials now also carry 8 annual fiscal years (income/balance/cash-flow via timeframe=annual), so the earnings hub gained Quarterly / Yearly tabs on both EPS &amp; Sales history and the Income statement (actuals only, chart removed). The 90% cap is unmoved because it reflects the missing estimate feed, not the actuals.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="46" t="inlineStr">
+      <c r="A25" s="50" t="inlineStr">
         <is>
           <t>R30</t>
         </is>
       </c>
-      <c r="B25" s="46" t="inlineStr">
+      <c r="B25" s="50" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="C25" s="46" t="inlineStr">
+      <c r="C25" s="50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D25" s="47" t="inlineStr">
+      <c r="D25" s="50" t="inlineStr">
         <is>
           <t>Screener sector/cap class + IPO recent perf + Macro regime label</t>
         </is>
       </c>
-      <c r="E25" s="47" t="inlineStr">
+      <c r="E25" s="50" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="F25" s="47" t="inlineStr">
+      <c r="F25" s="50" t="inlineStr">
         <is>
           <t>/v3/reference/tickers (class) + market_indices/market_breadth (regime)</t>
         </is>
       </c>
-      <c r="G25" s="47" t="inlineStr">
+      <c r="G25" s="50" t="inlineStr">
         <is>
           <t>Screener / IPOs / Macro · sector-cap class, IPO perf, regime label</t>
         </is>
       </c>
-      <c r="H25" s="46" t="inlineStr">
+      <c r="H25" s="50" t="inlineStr">
         <is>
           <t>100% ✅</t>
         </is>
       </c>
-      <c r="I25" s="47" t="inlineStr">
+      <c r="I25" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J25" s="47" t="inlineStr">
+      <c r="J25" s="50" t="inlineStr">
         <is>
           <t>⬆ 70% → 100% on 2026-07-23 — all 3 sub-parts done. ✅ Sector/cap classification live (companies). ✅ IPO aftermarket perf live (ipos.job, Polygon /v2/aggs). ✅ Macro regime label now computed: macro.tsx derives Risk-On / Neutral / Risk-Off by voting three live signals — VIX/VIXY level, market breadth (adv/dec from market_breadth) and the 10-year Treasury yield — replacing the hardcoded 'Risk-On Rally'. All Polygon/public data, no vendor purchase.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="44" t="inlineStr">
+      <c r="A26" s="49" t="inlineStr">
         <is>
           <t>R32</t>
         </is>
       </c>
-      <c r="B26" s="44" t="inlineStr">
+      <c r="B26" s="49" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="C26" s="44" t="inlineStr">
+      <c r="C26" s="49" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D26" s="45" t="inlineStr">
+      <c r="D26" s="49" t="inlineStr">
         <is>
           <t>Options Chain live (bid/ask/IV/OI/Greeks)</t>
         </is>
       </c>
-      <c r="E26" s="45" t="inlineStr">
+      <c r="E26" s="49" t="inlineStr">
         <is>
           <t>Polygon → Tradier</t>
         </is>
       </c>
-      <c r="F26" s="45" t="inlineStr">
+      <c r="F26" s="49" t="inlineStr">
         <is>
           <t>Polygon /v3/reference/options/contracts + /v2/aggs/ticker/O:{contract}/range/1/day/…; Tradier /v1/markets/options/chains (quotes — 🔴 unwired). Polygon /v3/snapshot/options → 403</t>
         </is>
       </c>
-      <c r="G26" s="45" t="inlineStr">
+      <c r="G26" s="49" t="inlineStr">
         <is>
           <t>Options · options chain</t>
         </is>
       </c>
-      <c r="H26" s="44" t="inlineStr">
+      <c r="H26" s="49" t="inlineStr">
         <is>
           <t>45% ⬆</t>
         </is>
       </c>
-      <c r="I26" s="45" t="inlineStr">
-        <is>
-          <t>Greeks, IV, open interest and bid/ask are still 🔴 hard-blocked — Polygon's options *snapshot* endpoint returns NOT_AUTHORIZED on the current plan (re-probed live 2026-07-22, still 403). Those four columns cannot be made real without a vendor purchase</t>
-        </is>
-      </c>
-      <c r="J26" s="45" t="inlineStr">
-        <is>
-          <t>⬆ Raised from 25%, but read the nuance — the block has NOT lifted. What changed is a different endpoint: option contract aggregates *are* authorized, so options-chains.job.ts now writes real per-contract OHLC, VWAP, trade count and range %. So the chain is no longer wholly synthetic — traded price/volume history per contract is genuine market data. But the quote-side surface a user actually reads an options chain for (bid/ask spread, IV, OI, greeks) is still fabricated. Unblock = Tradier (token already held, unwired) or Polygon Options Advanced</t>
+      <c r="I26" s="49" t="inlineStr">
+        <is>
+          <t>Greeks, IV, open interest and bid/ask are still 🔴 hard-blocked — Polygon's options snapshot endpoint returns NOT_AUTHORIZED on the current plan (re-probed live 2026-07-22, still 403). Those four columns cannot be made real without a vendor purchase</t>
+        </is>
+      </c>
+      <c r="J26" s="49" t="inlineStr">
+        <is>
+          <t>⬆ Raised from 25%, but read the nuance — the block has NOT lifted. What changed is a different endpoint: option contract aggregates are authorized, so options-chains.job.ts now writes real per-contract OHLC, VWAP, trade count and range %. So the chain is no longer wholly synthetic — traded price/volume history per contract is genuine market data. But the quote-side surface a user actually reads an options chain for (bid/ask spread, IV, OI, greeks) is still fabricated. Unblock = Tradier (token already held, unwired) or Polygon Options Advanced</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="46" t="inlineStr">
+      <c r="A27" s="50" t="inlineStr">
         <is>
           <t>R34</t>
         </is>
       </c>
-      <c r="B27" s="46" t="inlineStr">
+      <c r="B27" s="50" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="C27" s="46" t="inlineStr">
+      <c r="C27" s="50" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D27" s="47" t="inlineStr">
+      <c r="D27" s="50" t="inlineStr">
         <is>
           <t>ENABLER: AI service + ANTHROPIC key + prompt infra</t>
         </is>
       </c>
-      <c r="E27" s="47" t="inlineStr">
+      <c r="E27" s="50" t="inlineStr">
         <is>
           <t>Anthropic (deferred)</t>
         </is>
       </c>
-      <c r="F27" s="47" t="inlineStr">
+      <c r="F27" s="50" t="inlineStr">
         <is>
           <t>— (unwired by decision)</t>
         </is>
       </c>
-      <c r="G27" s="47" t="inlineStr">
-        <is>
-          <t>— *(AI enabler)*</t>
-        </is>
-      </c>
-      <c r="H27" s="46" t="inlineStr">
+      <c r="G27" s="50" t="inlineStr">
+        <is>
+          <t>— (AI enabler)</t>
+        </is>
+      </c>
+      <c r="H27" s="50" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="I27" s="47" t="inlineStr">
+      <c r="I27" s="50" t="inlineStr">
         <is>
           <t>AI service</t>
         </is>
       </c>
-      <c r="J27" s="47" t="inlineStr">
+      <c r="J27" s="50" t="inlineStr">
         <is>
           <t>⏸️ Deferred by decision (2026-07-21) — you chose labeled placeholders over wiring Anthropic this phase. Not blocked: ANTHROPIC_API_KEY is provisioned; this is a scope choice to avoid per-request LLM cost until later</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="44" t="inlineStr">
+      <c r="A28" s="49" t="inlineStr">
         <is>
           <t>R35</t>
         </is>
       </c>
-      <c r="B28" s="44" t="inlineStr">
+      <c r="B28" s="49" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="C28" s="44" t="inlineStr">
+      <c r="C28" s="49" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D28" s="45" t="inlineStr">
+      <c r="D28" s="49" t="inlineStr">
         <is>
           <t>Dashboard 'What Matters Now' AI card</t>
         </is>
       </c>
-      <c r="E28" s="45" t="inlineStr">
+      <c r="E28" s="49" t="inlineStr">
         <is>
           <t>Anthropic (deferred)</t>
         </is>
       </c>
-      <c r="F28" s="45" t="inlineStr">
+      <c r="F28" s="49" t="inlineStr">
         <is>
           <t>— (unwired by decision)</t>
         </is>
       </c>
-      <c r="G28" s="45" t="inlineStr">
+      <c r="G28" s="49" t="inlineStr">
         <is>
           <t>Dashboard · "What Matters Now" (AI — unwired)</t>
         </is>
       </c>
-      <c r="H28" s="44" t="inlineStr">
+      <c r="H28" s="49" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="I28" s="45" t="inlineStr">
+      <c r="I28" s="49" t="inlineStr">
         <is>
           <t>Real AI narrative</t>
         </is>
       </c>
-      <c r="J28" s="45" t="inlineStr">
+      <c r="J28" s="49" t="inlineStr">
         <is>
           <t>⏸️ Deferred by decision — card ships as a labeled placeholder; becomes real once R34 (Anthropic) is switched on</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="46" t="inlineStr">
+      <c r="A29" s="50" t="inlineStr">
         <is>
           <t>R36</t>
         </is>
       </c>
-      <c r="B29" s="46" t="inlineStr">
+      <c r="B29" s="50" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="C29" s="46" t="inlineStr">
+      <c r="C29" s="50" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D29" s="47" t="inlineStr">
+      <c r="D29" s="50" t="inlineStr">
         <is>
           <t>Recaps AI narrative</t>
         </is>
       </c>
-      <c r="E29" s="47" t="inlineStr">
+      <c r="E29" s="50" t="inlineStr">
         <is>
           <t>Anthropic (deferred)</t>
         </is>
       </c>
-      <c r="F29" s="47" t="inlineStr">
+      <c r="F29" s="50" t="inlineStr">
         <is>
           <t>— (unwired by decision)</t>
         </is>
       </c>
-      <c r="G29" s="47" t="inlineStr">
+      <c r="G29" s="50" t="inlineStr">
         <is>
           <t>Recap · AI narrative (unwired)</t>
         </is>
       </c>
-      <c r="H29" s="46" t="inlineStr">
+      <c r="H29" s="50" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="I29" s="47" t="inlineStr">
+      <c r="I29" s="50" t="inlineStr">
         <is>
           <t>Real AI narrative</t>
         </is>
       </c>
-      <c r="J29" s="47" t="inlineStr">
+      <c r="J29" s="50" t="inlineStr">
         <is>
           <t>⏸️ Deferred by decision (AI) + depends on R28 recap job (Milestone 3, in progress). Data layer will exist; only the LLM narrative is held back</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="44" t="inlineStr">
+      <c r="A30" s="49" t="inlineStr">
         <is>
           <t>R38</t>
         </is>
       </c>
-      <c r="B30" s="44" t="inlineStr">
+      <c r="B30" s="49" t="inlineStr">
         <is>
           <t>W8</t>
         </is>
       </c>
-      <c r="C30" s="44" t="inlineStr">
+      <c r="C30" s="49" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D30" s="45" t="inlineStr">
+      <c r="D30" s="49" t="inlineStr">
         <is>
           <t>Stock Detail AI (thesis/risk/confidence + technical analysis)</t>
         </is>
       </c>
-      <c r="E30" s="45" t="inlineStr">
+      <c r="E30" s="49" t="inlineStr">
         <is>
           <t>Anthropic (deferred)</t>
         </is>
       </c>
-      <c r="F30" s="45" t="inlineStr">
+      <c r="F30" s="49" t="inlineStr">
         <is>
           <t>— (unwired by decision)</t>
         </is>
       </c>
-      <c r="G30" s="45" t="inlineStr">
+      <c r="G30" s="49" t="inlineStr">
         <is>
           <t>Stock detail · AI thesis / risk (unwired)</t>
         </is>
       </c>
-      <c r="H30" s="44" t="inlineStr">
+      <c r="H30" s="49" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="I30" s="45" t="inlineStr">
+      <c r="I30" s="49" t="inlineStr">
         <is>
           <t>Real AI</t>
         </is>
       </c>
-      <c r="J30" s="45" t="inlineStr">
+      <c r="J30" s="49" t="inlineStr">
         <is>
           <t>⏸️ Deferred by decision — template text is honestly labeled 'AI-generated'; real model output awaits R34</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="46" t="inlineStr">
+      <c r="A31" s="50" t="inlineStr">
         <is>
           <t>R39</t>
         </is>
       </c>
-      <c r="B31" s="46" t="inlineStr">
+      <c r="B31" s="50" t="inlineStr">
         <is>
           <t>W8</t>
         </is>
       </c>
-      <c r="C31" s="46" t="inlineStr">
+      <c r="C31" s="50" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D31" s="47" t="inlineStr">
+      <c r="D31" s="50" t="inlineStr">
         <is>
           <t>Earnings+Analyst+Insider+Watchlist AI notes</t>
         </is>
       </c>
-      <c r="E31" s="47" t="inlineStr">
+      <c r="E31" s="50" t="inlineStr">
         <is>
           <t>Anthropic (deferred)</t>
         </is>
       </c>
-      <c r="F31" s="47" t="inlineStr">
+      <c r="F31" s="50" t="inlineStr">
         <is>
           <t>— (unwired by decision)</t>
         </is>
       </c>
-      <c r="G31" s="47" t="inlineStr">
+      <c r="G31" s="50" t="inlineStr">
         <is>
           <t>Earnings / Analyst / Insider / Watchlist · AI notes (unwired)</t>
         </is>
       </c>
-      <c r="H31" s="46" t="inlineStr">
+      <c r="H31" s="50" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="I31" s="47" t="inlineStr">
+      <c r="I31" s="50" t="inlineStr">
         <is>
           <t>Real AI</t>
         </is>
       </c>
-      <c r="J31" s="47" t="inlineStr">
+      <c r="J31" s="50" t="inlineStr">
         <is>
           <t>⏸️ Deferred by decision (AI). Includes R20 watchlist AI summary — non-AI watchlist parts already at 100%</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="44" t="inlineStr">
+      <c r="A32" s="49" t="inlineStr">
         <is>
           <t>R41</t>
         </is>
       </c>
-      <c r="B32" s="44" t="inlineStr">
+      <c r="B32" s="49" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="C32" s="44" t="inlineStr">
+      <c r="C32" s="49" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D32" s="45" t="inlineStr">
+      <c r="D32" s="49" t="inlineStr">
         <is>
           <t>Analyst Actions per-firm event table (upgrades/downgrades/PT)</t>
         </is>
       </c>
-      <c r="E32" s="45" t="inlineStr">
+      <c r="E32" s="49" t="inlineStr">
         <is>
           <t>Benzinga (🔴 403) / FMP</t>
         </is>
       </c>
-      <c r="F32" s="45" t="inlineStr">
+      <c r="F32" s="49" t="inlineStr">
         <is>
           <t>Benzinga /benzinga/v1/ratings → 403; FMP grades-consensus (snapshot only)</t>
         </is>
       </c>
-      <c r="G32" s="45" t="inlineStr">
+      <c r="G32" s="49" t="inlineStr">
         <is>
           <t>Analyst · per-firm event table</t>
         </is>
       </c>
-      <c r="H32" s="44" t="inlineStr">
+      <c r="H32" s="49" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="I32" s="45" t="inlineStr">
+      <c r="I32" s="49" t="inlineStr">
         <is>
           <t>Per-firm upgrade/downgrade events</t>
         </is>
       </c>
-      <c r="J32" s="45" t="inlineStr">
-        <is>
-          <t>🔴 Vendor-blocked, not effort — per-firm actions need Benzinga (403 on current plan). FMP gives only a consensus snapshot; Finnhub gives rating *history* but not per-firm. Requires a paid vendor decision</t>
+      <c r="J32" s="49" t="inlineStr">
+        <is>
+          <t>🔴 Vendor-blocked, not effort — per-firm actions need Benzinga (403 on current plan). FMP gives only a consensus snapshot; Finnhub gives rating history but not per-firm. Requires a paid vendor decision</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="46" t="inlineStr">
+      <c r="A33" s="50" t="inlineStr">
         <is>
           <t>R42</t>
         </is>
       </c>
-      <c r="B33" s="46" t="inlineStr">
+      <c r="B33" s="50" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="C33" s="46" t="inlineStr">
+      <c r="C33" s="50" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D33" s="47" t="inlineStr">
+      <c r="D33" s="50" t="inlineStr">
         <is>
           <t>Earnings depth (guidance/reaction/real-time actuals + tags)</t>
         </is>
       </c>
-      <c r="E33" s="47" t="inlineStr">
+      <c r="E33" s="50" t="inlineStr">
         <is>
           <t>FMP + Benzinga (🔴 403)</t>
         </is>
       </c>
-      <c r="F33" s="47" t="inlineStr">
+      <c r="F33" s="50" t="inlineStr">
         <is>
           <t>FMP /stable/earnings-calendar; Benzinga /benzinga/v1/{earnings,guidance} → 403; reaction derivable from ohlcv_bars</t>
         </is>
       </c>
-      <c r="G33" s="47" t="inlineStr">
+      <c r="G33" s="50" t="inlineStr">
         <is>
           <t>Earnings hub · guidance / reaction depth</t>
         </is>
       </c>
-      <c r="H33" s="46" t="inlineStr">
+      <c r="H33" s="50" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="I33" s="47" t="inlineStr">
+      <c r="I33" s="50" t="inlineStr">
         <is>
           <t>Guidance + price reaction</t>
         </is>
       </c>
-      <c r="J33" s="47" t="inlineStr">
+      <c r="J33" s="50" t="inlineStr">
         <is>
           <t>🟠 Partially unblockable now — session (BMO/AMC) IS available on the held Finnhub key (unwired); guidance/reaction still need a Benzinga-class feed. Reaction could also be computed from ohlcv_bars post-print</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="44" t="inlineStr">
+      <c r="A34" s="49" t="inlineStr">
         <is>
           <t>R43</t>
         </is>
       </c>
-      <c r="B34" s="44" t="inlineStr">
+      <c r="B34" s="49" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="C34" s="44" t="inlineStr">
+      <c r="C34" s="49" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D34" s="45" t="inlineStr">
+      <c r="D34" s="49" t="inlineStr">
         <is>
           <t>Options flow + dark-pool prints</t>
         </is>
       </c>
-      <c r="E34" s="45" t="inlineStr">
+      <c r="E34" s="49" t="inlineStr">
         <is>
           <t>Unusual Whales (not subscribed)</t>
         </is>
       </c>
-      <c r="F34" s="45" t="inlineStr">
+      <c r="F34" s="49" t="inlineStr">
         <is>
           <t>— (unwired)</t>
         </is>
       </c>
-      <c r="G34" s="45" t="inlineStr">
+      <c r="G34" s="49" t="inlineStr">
         <is>
           <t>Options · flow + dark-pool prints</t>
         </is>
       </c>
-      <c r="H34" s="44" t="inlineStr">
+      <c r="H34" s="49" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="I34" s="45" t="inlineStr">
+      <c r="I34" s="49" t="inlineStr">
         <is>
           <t>Entire feature</t>
         </is>
       </c>
-      <c r="J34" s="45" t="inlineStr">
+      <c r="J34" s="49" t="inlineStr">
         <is>
           <t>🔴 Vendor-blocked — needs a UnusualWhales / Polygon-paid flow add-on the current plans don't include. Marked P2 (post-MVP) in the plan itself</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="46" t="inlineStr">
+      <c r="A35" s="50" t="inlineStr">
         <is>
           <t>R44</t>
         </is>
       </c>
-      <c r="B35" s="46" t="inlineStr">
+      <c r="B35" s="50" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="C35" s="46" t="inlineStr">
+      <c r="C35" s="50" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D35" s="47" t="inlineStr">
+      <c r="D35" s="50" t="inlineStr">
         <is>
           <t>Alerts engine (12 alert types + watchlist toggles)</t>
         </is>
       </c>
-      <c r="E35" s="47" t="inlineStr">
+      <c r="E35" s="50" t="inlineStr">
         <is>
           <t>— (internal)</t>
         </is>
       </c>
-      <c r="F35" s="47" t="inlineStr">
+      <c r="F35" s="50" t="inlineStr">
         <is>
           <t>— (rules over synced Firestore data)</t>
         </is>
       </c>
-      <c r="G35" s="47" t="inlineStr">
+      <c r="G35" s="50" t="inlineStr">
         <is>
           <t>Alerts · alerts engine (screen not built)</t>
         </is>
       </c>
-      <c r="H35" s="46" t="inlineStr">
+      <c r="H35" s="50" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="I35" s="47" t="inlineStr">
+      <c r="I35" s="50" t="inlineStr">
         <is>
           <t>Rules engine + 12 alert types</t>
         </is>
       </c>
-      <c r="J35" s="47" t="inlineStr">
+      <c r="J35" s="50" t="inlineStr">
         <is>
           <t>🔨 Not built — no blocker. Net-new backend (evaluate rules against synced data, per-user toggles, delivery). All input data exists; it is buildable now, just not yet scheduled (W9)</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="44" t="inlineStr">
+      <c r="A36" s="49" t="inlineStr">
         <is>
           <t>R46</t>
         </is>
       </c>
-      <c r="B36" s="44" t="inlineStr">
+      <c r="B36" s="49" t="inlineStr">
         <is>
           <t>W10</t>
         </is>
       </c>
-      <c r="C36" s="44" t="inlineStr">
+      <c r="C36" s="49" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D36" s="45" t="inlineStr">
+      <c r="D36" s="49" t="inlineStr">
         <is>
           <t>Editorial + dropped-feature decisions</t>
         </is>
       </c>
-      <c r="E36" s="45" t="inlineStr">
+      <c r="E36" s="49" t="inlineStr">
         <is>
           <t>— (product)</t>
         </is>
       </c>
-      <c r="F36" s="45" t="inlineStr">
+      <c r="F36" s="49" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G36" s="45" t="inlineStr">
-        <is>
-          <t>— *(product decisions)*</t>
-        </is>
-      </c>
-      <c r="H36" s="44" t="inlineStr">
+      <c r="G36" s="49" t="inlineStr">
+        <is>
+          <t>— (product decisions)</t>
+        </is>
+      </c>
+      <c r="H36" s="49" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="I36" s="45" t="inlineStr">
+      <c r="I36" s="49" t="inlineStr">
         <is>
           <t>Product decisions</t>
         </is>
       </c>
-      <c r="J36" s="45" t="inlineStr">
+      <c r="J36" s="49" t="inlineStr">
         <is>
           <t>🗓️ W10 by design — a decision/curation task (which themes, presets, sections to keep or cut), correctly sequenced for launch week; not an engineering gap</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="46" t="inlineStr">
+      <c r="A37" s="50" t="inlineStr">
         <is>
           <t>R47</t>
         </is>
       </c>
-      <c r="B37" s="46" t="inlineStr">
+      <c r="B37" s="50" t="inlineStr">
         <is>
           <t>W10</t>
         </is>
       </c>
-      <c r="C37" s="46" t="inlineStr">
+      <c r="C37" s="50" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D37" s="47" t="inlineStr">
+      <c r="D37" s="50" t="inlineStr">
         <is>
           <t>Earnings + Macro calendars on real date ranges (structural)</t>
         </is>
       </c>
-      <c r="E37" s="47" t="inlineStr">
+      <c r="E37" s="50" t="inlineStr">
         <is>
           <t>FMP + Finnhub</t>
         </is>
       </c>
-      <c r="F37" s="47" t="inlineStr">
+      <c r="F37" s="50" t="inlineStr">
         <is>
           <t>FMP /stable/earnings-calendar; Finnhub /calendar/economic</t>
         </is>
       </c>
-      <c r="G37" s="47" t="inlineStr">
+      <c r="G37" s="50" t="inlineStr">
         <is>
           <t>Earnings + Macro calendars · date-anchored calendars</t>
         </is>
       </c>
-      <c r="H37" s="46" t="inlineStr">
+      <c r="H37" s="50" t="inlineStr">
         <is>
           <t>80%</t>
         </is>
       </c>
-      <c r="I37" s="47" t="inlineStr">
+      <c r="I37" s="50" t="inlineStr">
         <is>
           <t>Earnings coverage thin</t>
         </is>
       </c>
-      <c r="J37" s="47" t="inlineStr">
+      <c r="J37" s="50" t="inlineStr">
         <is>
           <t>Ahead of schedule — date-anchored calendar built (earnings-calendar.tsx, calendar-range.ts); FMP's 10-row coverage limits it</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="44" t="inlineStr">
+      <c r="A38" s="49" t="inlineStr">
         <is>
           <t>R48</t>
         </is>
       </c>
-      <c r="B38" s="44" t="inlineStr">
+      <c r="B38" s="49" t="inlineStr">
         <is>
           <t>W10</t>
         </is>
       </c>
-      <c r="C38" s="44" t="inlineStr">
+      <c r="C38" s="49" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D38" s="45" t="inlineStr">
+      <c r="D38" s="49" t="inlineStr">
         <is>
           <t>Full regression + empty-states + mobile + performance</t>
         </is>
       </c>
-      <c r="E38" s="45" t="inlineStr">
+      <c r="E38" s="49" t="inlineStr">
         <is>
           <t>— (QA)</t>
         </is>
       </c>
-      <c r="F38" s="45" t="inlineStr">
+      <c r="F38" s="49" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G38" s="45" t="inlineStr">
-        <is>
-          <t>— *(QA)*</t>
-        </is>
-      </c>
-      <c r="H38" s="44" t="inlineStr">
+      <c r="G38" s="49" t="inlineStr">
+        <is>
+          <t>— (QA)</t>
+        </is>
+      </c>
+      <c r="H38" s="49" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="I38" s="45" t="inlineStr">
+      <c r="I38" s="49" t="inlineStr">
         <is>
           <t>QA gate</t>
         </is>
       </c>
-      <c r="J38" s="45" t="inlineStr">
+      <c r="J38" s="49" t="inlineStr">
         <is>
           <t>🗓️ W10 by design — final QA/regression gate, only meaningful once features stop changing. Partially advanced by R21 empty-state work</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="46" t="inlineStr">
+      <c r="A39" s="50" t="inlineStr">
         <is>
           <t>R49</t>
         </is>
       </c>
-      <c r="B39" s="46" t="inlineStr">
+      <c r="B39" s="50" t="inlineStr">
         <is>
           <t>W10</t>
         </is>
       </c>
-      <c r="C39" s="46" t="inlineStr">
+      <c r="C39" s="50" t="inlineStr">
         <is>
           <t>🔵</t>
         </is>
       </c>
-      <c r="D39" s="47" t="inlineStr">
+      <c r="D39" s="50" t="inlineStr">
         <is>
           <t>Security review + launch checklist</t>
         </is>
       </c>
-      <c r="E39" s="47" t="inlineStr">
+      <c r="E39" s="50" t="inlineStr">
         <is>
           <t>— (security)</t>
         </is>
       </c>
-      <c r="F39" s="47" t="inlineStr">
+      <c r="F39" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G39" s="47" t="inlineStr">
-        <is>
-          <t>— *(security)*</t>
-        </is>
-      </c>
-      <c r="H39" s="46" t="inlineStr">
+      <c r="G39" s="50" t="inlineStr">
+        <is>
+          <t>— (security)</t>
+        </is>
+      </c>
+      <c r="H39" s="50" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="I39" s="47" t="inlineStr">
+      <c r="I39" s="50" t="inlineStr">
         <is>
           <t>Full review + checklist</t>
         </is>
       </c>
-      <c r="J39" s="47" t="inlineStr">
+      <c r="J39" s="50" t="inlineStr">
         <is>
           <t>🗓️ W10 by design. Already done ahead: runtime SA least-privilege; Firestore rules server-write-only; retention module; 2026-07-22 rules hardening — plans writable by admin on featureFlags+updatedAt only (a client that could rewrite amount could set a plan to $0), create/delete denied; feature_adoption is the only client-writable analytics collection and is constrained (row must belong to caller, openCount may only increase, ownership immutable, delete denied); adminDashboard/userManagement are staff-only on every plan so they can never be sold (privilege escalation). ⚠️ Still outstanding, all three real: (1) POLYGON_API_KEY is still un-rotated (exposed in chat; Secret Manager version 4 enabled; deploy/rotate-polygon-key.sh automates all of it except generating the replacement). (2) ✅ Resolved 2026-07-23 without the risky rewrite. Backend reachability was delivered by a SEPARATE public service (market-catalyst-live, APP_ROLE=live) that mounts only LiveModule — /sync, /purge, /retention, /admin all return 404 there (verified) while the worker stays --no-allow-unauthenticated with ADMIN_GUARD_TRUST_IAM=true. No Hosting→Cloud Run rewrite was used, so the world-callable-admin risk never materialised. (3) Both repos ship a firestore.rules and they have drifted — the live ruleset deploys from MarketCatalystUI/firestore.rules; the backend copy is stale and now carries a DO-NOT-DEPLOY header</t>
         </is>
@@ -4740,4 +4786,620 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" style="27" min="1" max="1"/>
+    <col width="42" customWidth="1" style="27" min="2" max="2"/>
+    <col width="12" customWidth="1" style="27" min="3" max="3"/>
+    <col width="26" customWidth="1" style="27" min="4" max="4"/>
+    <col width="46" customWidth="1" style="27" min="5" max="5"/>
+    <col width="34" customWidth="1" style="27" min="6" max="6"/>
+    <col width="30" customWidth="1" style="27" min="7" max="7"/>
+    <col width="34" customWidth="1" style="27" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>MarketCatalyst — Path to 100% (2026-07-29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="90" customHeight="1" s="27">
+      <c r="A2" s="51" t="inlineStr">
+        <is>
+          <t>Path to 100% overall, in one paragraph: two moves are free and close five rows outright (R44 alerts engine, R49 key rotation) plus meaningfully advance two more (R32 via Tradier, R42's session/reaction half) with zero new spend. The single highest-leverage remaining decision is reversing the AI deferral (R34) — the key is already provisioned and it unblocks 5 rows at 0% simultaneously. Everything else (R29 estimates, R41 analyst events, R42's guidance half, R43 options flow) is a vendor-purchase decision, not an effort gap — no amount of engineering time closes them without buying Benzinga / Unusual Whales / a Polygon add-on. R46/R48 are deliberately sequenced last (launch-week gates) and need no unblocking, just to be reached in order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t>Row</t>
+        </is>
+      </c>
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>Current %</t>
+        </is>
+      </c>
+      <c r="D4" s="52" t="inlineStr">
+        <is>
+          <t>Gap type</t>
+        </is>
+      </c>
+      <c r="E4" s="52" t="inlineStr">
+        <is>
+          <t>What closes it</t>
+        </is>
+      </c>
+      <c r="F4" s="52" t="inlineStr">
+        <is>
+          <t>Cost/decision needed</t>
+        </is>
+      </c>
+      <c r="G4" s="52" t="inlineStr">
+        <is>
+          <t>Effort if unblocked</t>
+        </is>
+      </c>
+      <c r="H4" s="52" t="inlineStr">
+        <is>
+          <t>Recommended order</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="53" t="inlineStr">
+        <is>
+          <t>R44</t>
+        </is>
+      </c>
+      <c r="B5" s="53" t="inlineStr">
+        <is>
+          <t>Alerts engine (12 alert types + watchlist toggles)</t>
+        </is>
+      </c>
+      <c r="C5" s="53" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="D5" s="53" t="inlineStr">
+        <is>
+          <t>Buildable now — no blocker</t>
+        </is>
+      </c>
+      <c r="E5" s="53" t="inlineStr">
+        <is>
+          <t>Build the rules engine over already-synced Firestore data + per-user toggles + delivery (email/in-app). All input data already exists.</t>
+        </is>
+      </c>
+      <c r="F5" s="53" t="inlineStr">
+        <is>
+          <t>None — engineering time only</t>
+        </is>
+      </c>
+      <c r="G5" s="53" t="inlineStr">
+        <is>
+          <t>~3.5 person-days (per original plan)</t>
+        </is>
+      </c>
+      <c r="H5" s="53" t="inlineStr">
+        <is>
+          <t>1 — do first, zero cost, closes a whole row</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="53" t="inlineStr">
+        <is>
+          <t>R49</t>
+        </is>
+      </c>
+      <c r="B6" s="53" t="inlineStr">
+        <is>
+          <t>Security review + launch checklist</t>
+        </is>
+      </c>
+      <c r="C6" s="53" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="D6" s="53" t="inlineStr">
+        <is>
+          <t>Buildable now — no blocker</t>
+        </is>
+      </c>
+      <c r="E6" s="53" t="inlineStr">
+        <is>
+          <t>Rotate POLYGON_API_KEY (script exists, just run it — the only manual step is generating the replacement key at the vendor dashboard); finish the launch checklist.</t>
+        </is>
+      </c>
+      <c r="F6" s="53" t="inlineStr">
+        <is>
+          <t>None — 15 minutes of vendor-dashboard clicking + checklist time</t>
+        </is>
+      </c>
+      <c r="G6" s="53" t="inlineStr">
+        <is>
+          <t>~1 person-day remaining</t>
+        </is>
+      </c>
+      <c r="H6" s="53" t="inlineStr">
+        <is>
+          <t>2 — closes a live credential-exposure risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="53" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B7" s="53" t="inlineStr">
+        <is>
+          <t>Options Chain live (bid/ask/IV/OI/Greeks)</t>
+        </is>
+      </c>
+      <c r="C7" s="53" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+      <c r="D7" s="53" t="inlineStr">
+        <is>
+          <t>Buildable now (partial) — token already held</t>
+        </is>
+      </c>
+      <c r="E7" s="53" t="inlineStr">
+        <is>
+          <t>Wire Tradier — the access token is already provisioned and unwired. Closes bid/ask/IV/OI/Greeks without any new purchase.</t>
+        </is>
+      </c>
+      <c r="F7" s="53" t="inlineStr">
+        <is>
+          <t>None if Tradier's free tier suffices; Polygon Options Advanced is the paid fallback</t>
+        </is>
+      </c>
+      <c r="G7" s="53" t="inlineStr">
+        <is>
+          <t>~2-3 person-days to wire + test</t>
+        </is>
+      </c>
+      <c r="H7" s="53" t="inlineStr">
+        <is>
+          <t>3 — biggest 'free' unlock left</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="53" t="inlineStr">
+        <is>
+          <t>R42</t>
+        </is>
+      </c>
+      <c r="B8" s="53" t="inlineStr">
+        <is>
+          <t>Earnings depth (guidance/reaction/real-time actuals + tags)</t>
+        </is>
+      </c>
+      <c r="C8" s="53" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="D8" s="53" t="inlineStr">
+        <is>
+          <t>Buildable now (partial) — key already held</t>
+        </is>
+      </c>
+      <c r="E8" s="53" t="inlineStr">
+        <is>
+          <t>Wire Finnhub's earnings-calendar session field (BMO/AMC) — key already held, currently unused. Reaction is computable from ohlcv_bars post-print without any vendor.</t>
+        </is>
+      </c>
+      <c r="F8" s="53" t="inlineStr">
+        <is>
+          <t>None for session+reaction; guidance still needs a Benzinga-class feed (see below)</t>
+        </is>
+      </c>
+      <c r="G8" s="53" t="inlineStr">
+        <is>
+          <t>~1 person-day for session+reaction</t>
+        </is>
+      </c>
+      <c r="H8" s="53" t="inlineStr">
+        <is>
+          <t>4 — partial close, no cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="54" t="inlineStr">
+        <is>
+          <t>R34 / R35 / R36 / R38 / R39</t>
+        </is>
+      </c>
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t>AI enabler + What Matters Now + Recaps narrative + Stock Detail AI + Earnings/Analyst/Insider/Watchlist AI notes (5 rows)</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>0% each</t>
+        </is>
+      </c>
+      <c r="D9" s="54" t="inlineStr">
+        <is>
+          <t>Deferred by decision, not blocked</t>
+        </is>
+      </c>
+      <c r="E9" s="54" t="inlineStr">
+        <is>
+          <t>Reverse the 2026-07-21 decision to defer Anthropic. ANTHROPIC_API_KEY is already provisioned; wiring R34 (the enabler) unlocks all 4 dependent rows.</t>
+        </is>
+      </c>
+      <c r="F9" s="54" t="inlineStr">
+        <is>
+          <t>Anthropic API usage cost (per-request LLM spend) — a budget decision, not a purchase-approval one</t>
+        </is>
+      </c>
+      <c r="G9" s="54" t="inlineStr">
+        <is>
+          <t>~2.5 + 2 + 3 + 5 + 5 = ~17.5 person-days total (per original plan)</t>
+        </is>
+      </c>
+      <c r="H9" s="54" t="inlineStr">
+        <is>
+          <t>5 — single highest-leverage decision on the whole board (5 rows, 0%→100% once made)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="55" t="inlineStr">
+        <is>
+          <t>R29</t>
+        </is>
+      </c>
+      <c r="B10" s="55" t="inlineStr">
+        <is>
+          <t>10-quarter EPS history — estimates half</t>
+        </is>
+      </c>
+      <c r="C10" s="55" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="D10" s="55" t="inlineStr">
+        <is>
+          <t>Vendor-blocked</t>
+        </is>
+      </c>
+      <c r="E10" s="55" t="inlineStr">
+        <is>
+          <t>Purchase Polygon's Benzinga Earnings &amp; Estimates add-on. Actuals are already 100% Polygon and done; only the forward-estimate overlay is missing.</t>
+        </is>
+      </c>
+      <c r="F10" s="55" t="inlineStr">
+        <is>
+          <t>Paid add-on to the existing Polygon plan</t>
+        </is>
+      </c>
+      <c r="G10" s="55" t="inlineStr">
+        <is>
+          <t>Wiring is small once purchased (data already flows through the same job)</t>
+        </is>
+      </c>
+      <c r="H10" s="55" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="55" t="inlineStr">
+        <is>
+          <t>R41</t>
+        </is>
+      </c>
+      <c r="B11" s="55" t="inlineStr">
+        <is>
+          <t>Analyst Actions per-firm event table</t>
+        </is>
+      </c>
+      <c r="C11" s="55" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="D11" s="55" t="inlineStr">
+        <is>
+          <t>Vendor-blocked</t>
+        </is>
+      </c>
+      <c r="E11" s="55" t="inlineStr">
+        <is>
+          <t>Purchase Benzinga (via Polygon add-on or direct). FMP only gives a consensus snapshot, Finnhub only gives rating history — neither has per-firm events.</t>
+        </is>
+      </c>
+      <c r="F11" s="55" t="inlineStr">
+        <is>
+          <t>Paid vendor (Benzinga)</t>
+        </is>
+      </c>
+      <c r="G11" s="55" t="inlineStr">
+        <is>
+          <t>~4.5 person-days once the feed exists (per original plan)</t>
+        </is>
+      </c>
+      <c r="H11" s="55" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="55" t="inlineStr">
+        <is>
+          <t>R42</t>
+        </is>
+      </c>
+      <c r="B12" s="55" t="inlineStr">
+        <is>
+          <t>Earnings depth — guidance half</t>
+        </is>
+      </c>
+      <c r="C12" s="55" t="inlineStr">
+        <is>
+          <t>(same row as above)</t>
+        </is>
+      </c>
+      <c r="D12" s="55" t="inlineStr">
+        <is>
+          <t>Vendor-blocked</t>
+        </is>
+      </c>
+      <c r="E12" s="55" t="inlineStr">
+        <is>
+          <t>Same Benzinga-class feed as R41/R29 — bundle this purchase decision with those two.</t>
+        </is>
+      </c>
+      <c r="F12" s="55" t="inlineStr">
+        <is>
+          <t>Paid vendor (Benzinga)</t>
+        </is>
+      </c>
+      <c r="G12" s="55" t="inlineStr">
+        <is>
+          <t>small, rides along with R41</t>
+        </is>
+      </c>
+      <c r="H12" s="55" t="inlineStr">
+        <is>
+          <t>7 (bundle with R41/R29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="55" t="inlineStr">
+        <is>
+          <t>R43</t>
+        </is>
+      </c>
+      <c r="B13" s="55" t="inlineStr">
+        <is>
+          <t>Options flow + dark-pool prints</t>
+        </is>
+      </c>
+      <c r="C13" s="55" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="D13" s="55" t="inlineStr">
+        <is>
+          <t>Vendor-blocked</t>
+        </is>
+      </c>
+      <c r="E13" s="55" t="inlineStr">
+        <is>
+          <t>Purchase Unusual Whales or the Polygon-paid flow add-on. Explicitly marked P2/post-MVP in the original plan.</t>
+        </is>
+      </c>
+      <c r="F13" s="55" t="inlineStr">
+        <is>
+          <t>Paid vendor (Unusual Whales or Polygon flow add-on)</t>
+        </is>
+      </c>
+      <c r="G13" s="55" t="inlineStr">
+        <is>
+          <t>~2.5 person-days once the feed exists (per original plan)</t>
+        </is>
+      </c>
+      <c r="H13" s="55" t="inlineStr">
+        <is>
+          <t>8 — lowest priority vendor purchase, P2 by design</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="55" t="inlineStr">
+        <is>
+          <t>R47</t>
+        </is>
+      </c>
+      <c r="B14" s="55" t="inlineStr">
+        <is>
+          <t>Earnings + Macro calendars on real date ranges</t>
+        </is>
+      </c>
+      <c r="C14" s="55" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
+      <c r="D14" s="55" t="inlineStr">
+        <is>
+          <t>Partially vendor-limited</t>
+        </is>
+      </c>
+      <c r="E14" s="55" t="inlineStr">
+        <is>
+          <t>Structural work is done and ahead of schedule; remaining gap is FMP's 10-row calendar coverage ceiling. Revisit only if a richer calendar vendor is purchased for R41/R29 anyway.</t>
+        </is>
+      </c>
+      <c r="F14" s="55" t="inlineStr">
+        <is>
+          <t>None required now; a bonus if the Benzinga purchase above happens</t>
+        </is>
+      </c>
+      <c r="G14" s="55" t="inlineStr">
+        <is>
+          <t>Small, incremental</t>
+        </is>
+      </c>
+      <c r="H14" s="55" t="inlineStr">
+        <is>
+          <t>9 — opportunistic, not urgent</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="55" t="inlineStr">
+        <is>
+          <t>R46</t>
+        </is>
+      </c>
+      <c r="B15" s="55" t="inlineStr">
+        <is>
+          <t>Editorial + dropped-feature decisions</t>
+        </is>
+      </c>
+      <c r="C15" s="55" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="D15" s="55" t="inlineStr">
+        <is>
+          <t>Launch-week gate, by design</t>
+        </is>
+      </c>
+      <c r="E15" s="55" t="inlineStr">
+        <is>
+          <t>Product decision task (which themes/presets/sections to keep or cut). Not an engineering gap — sequence it in W10 as planned.</t>
+        </is>
+      </c>
+      <c r="F15" s="55" t="inlineStr">
+        <is>
+          <t>None — product time only</t>
+        </is>
+      </c>
+      <c r="G15" s="55" t="inlineStr">
+        <is>
+          <t>~3 person-days (per original plan)</t>
+        </is>
+      </c>
+      <c r="H15" s="55" t="inlineStr">
+        <is>
+          <t>10 — correctly sequenced last</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="55" t="inlineStr">
+        <is>
+          <t>R48</t>
+        </is>
+      </c>
+      <c r="B16" s="55" t="inlineStr">
+        <is>
+          <t>Full regression + empty-states + mobile + performance</t>
+        </is>
+      </c>
+      <c r="C16" s="55" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="D16" s="55" t="inlineStr">
+        <is>
+          <t>Launch-week gate, by design</t>
+        </is>
+      </c>
+      <c r="E16" s="55" t="inlineStr">
+        <is>
+          <t>Final QA/regression pass. Only meaningful once feature work (rows above) has actually stopped changing — don't start early.</t>
+        </is>
+      </c>
+      <c r="F16" s="55" t="inlineStr">
+        <is>
+          <t>None — QA time only</t>
+        </is>
+      </c>
+      <c r="G16" s="55" t="inlineStr">
+        <is>
+          <t>~4 person-days (per original plan)</t>
+        </is>
+      </c>
+      <c r="H16" s="55" t="inlineStr">
+        <is>
+          <t>11 — correctly sequenced last</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="40" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="56" t="inlineStr">
+        <is>
+          <t>Green = zero-cost, buildable now</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="57" t="inlineStr">
+        <is>
+          <t>Amber = budget/scope decision (key already provisioned)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="58" t="inlineStr">
+        <is>
+          <t>Pink = vendor purchase required</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>